<commit_message>
chore: sync GST statistics files 2026-07-01
</commit_message>
<xml_diff>
--- a/gstdatabase/GSTR-1-2017-2018.xlsx
+++ b/gstdatabase/GSTR-1-2017-2018.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GSTN\Krishnan Sir\Monthly Report\Feb-26\GST Statistics Downloads 28th Feb 26\Downloads\GSTR 1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GSTN\Krishnan Sir\Monthly Report\May-26\GST Statistics Downloads 31st May 26\Downloads\GSTR 1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2F7782F-3CEB-43BD-9450-16AD877D56E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7772CF6D-528E-4F6F-A313-92E513D4D3FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -182,10 +182,10 @@
     <t>Andaman and Nicobar Islands</t>
   </si>
   <si>
-    <t>Data Considered upto 28th Feb 2026</t>
+    <t>Data Considered upto 31st May 2026</t>
   </si>
   <si>
-    <t>Filing %age as on 28th Feb 2026</t>
+    <t>Filing %age as on 31st May 2026</t>
   </si>
 </sst>
 </file>
@@ -374,15 +374,6 @@
       <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="17" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -396,6 +387,15 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="17" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -736,10 +736,10 @@
       <c r="L2" s="8"/>
     </row>
     <row r="3" spans="1:48" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="24" t="s">
+      <c r="A3" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="24"/>
+      <c r="B3" s="29"/>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -766,86 +766,86 @@
       <c r="L4" s="8"/>
     </row>
     <row r="5" spans="1:48" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A5" s="24" t="s">
+      <c r="A5" s="29" t="s">
         <v>48</v>
       </c>
-      <c r="B5" s="24"/>
-      <c r="C5" s="24"/>
+      <c r="B5" s="29"/>
+      <c r="C5" s="29"/>
     </row>
     <row r="7" spans="1:48" s="17" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A7" s="25" t="s">
+      <c r="A7" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="B7" s="26" t="s">
+      <c r="B7" s="31" t="s">
         <v>3</v>
       </c>
-      <c r="C7" s="27">
+      <c r="C7" s="24">
         <v>42917</v>
       </c>
-      <c r="D7" s="27"/>
-      <c r="E7" s="27"/>
-      <c r="F7" s="27"/>
-      <c r="G7" s="27"/>
-      <c r="H7" s="31">
+      <c r="D7" s="24"/>
+      <c r="E7" s="24"/>
+      <c r="F7" s="24"/>
+      <c r="G7" s="24"/>
+      <c r="H7" s="28">
         <v>42948</v>
       </c>
-      <c r="I7" s="31"/>
-      <c r="J7" s="31"/>
-      <c r="K7" s="31"/>
-      <c r="L7" s="31"/>
-      <c r="M7" s="27">
+      <c r="I7" s="28"/>
+      <c r="J7" s="28"/>
+      <c r="K7" s="28"/>
+      <c r="L7" s="28"/>
+      <c r="M7" s="24">
         <v>42979</v>
       </c>
-      <c r="N7" s="28"/>
-      <c r="O7" s="28"/>
-      <c r="P7" s="28"/>
-      <c r="Q7" s="28"/>
-      <c r="R7" s="31">
+      <c r="N7" s="25"/>
+      <c r="O7" s="25"/>
+      <c r="P7" s="25"/>
+      <c r="Q7" s="25"/>
+      <c r="R7" s="28">
         <v>43009</v>
       </c>
-      <c r="S7" s="31"/>
-      <c r="T7" s="31"/>
-      <c r="U7" s="31"/>
-      <c r="V7" s="31"/>
-      <c r="W7" s="27">
+      <c r="S7" s="28"/>
+      <c r="T7" s="28"/>
+      <c r="U7" s="28"/>
+      <c r="V7" s="28"/>
+      <c r="W7" s="24">
         <v>43040</v>
       </c>
-      <c r="X7" s="28"/>
-      <c r="Y7" s="28"/>
-      <c r="Z7" s="28"/>
-      <c r="AA7" s="28"/>
-      <c r="AB7" s="31">
+      <c r="X7" s="25"/>
+      <c r="Y7" s="25"/>
+      <c r="Z7" s="25"/>
+      <c r="AA7" s="25"/>
+      <c r="AB7" s="28">
         <v>43070</v>
       </c>
-      <c r="AC7" s="31"/>
-      <c r="AD7" s="31"/>
-      <c r="AE7" s="31"/>
-      <c r="AF7" s="31"/>
-      <c r="AG7" s="27">
+      <c r="AC7" s="28"/>
+      <c r="AD7" s="28"/>
+      <c r="AE7" s="28"/>
+      <c r="AF7" s="28"/>
+      <c r="AG7" s="24">
         <v>43101</v>
       </c>
-      <c r="AH7" s="28"/>
-      <c r="AI7" s="28"/>
-      <c r="AJ7" s="28"/>
-      <c r="AK7" s="28"/>
-      <c r="AL7" s="31">
+      <c r="AH7" s="25"/>
+      <c r="AI7" s="25"/>
+      <c r="AJ7" s="25"/>
+      <c r="AK7" s="25"/>
+      <c r="AL7" s="28">
         <v>43132</v>
       </c>
-      <c r="AM7" s="31"/>
-      <c r="AN7" s="31"/>
-      <c r="AO7" s="31"/>
-      <c r="AP7" s="31"/>
-      <c r="AQ7" s="27">
+      <c r="AM7" s="28"/>
+      <c r="AN7" s="28"/>
+      <c r="AO7" s="28"/>
+      <c r="AP7" s="28"/>
+      <c r="AQ7" s="24">
         <v>43160</v>
       </c>
-      <c r="AR7" s="28"/>
-      <c r="AS7" s="28"/>
-      <c r="AT7" s="28"/>
-      <c r="AU7" s="28"/>
+      <c r="AR7" s="25"/>
+      <c r="AS7" s="25"/>
+      <c r="AT7" s="25"/>
+      <c r="AU7" s="25"/>
     </row>
     <row r="8" spans="1:48" s="17" customFormat="1" ht="46.8" x14ac:dyDescent="0.3">
-      <c r="A8" s="25"/>
-      <c r="B8" s="26"/>
+      <c r="A8" s="30"/>
+      <c r="B8" s="31"/>
       <c r="C8" s="18" t="s">
         <v>4</v>
       </c>
@@ -1320,14 +1320,14 @@
       </c>
       <c r="E11" s="9">
         <f t="shared" si="0"/>
-        <v>22956</v>
+        <v>22958</v>
       </c>
       <c r="F11" s="22">
-        <v>207101</v>
+        <v>207103</v>
       </c>
       <c r="G11" s="10">
         <f t="shared" si="1"/>
-        <v>0.93801690324567677</v>
+        <v>0.93802596179105557</v>
       </c>
       <c r="H11" s="6">
         <v>86189</v>
@@ -1337,14 +1337,14 @@
       </c>
       <c r="J11" s="9">
         <f t="shared" si="2"/>
-        <v>2399</v>
+        <v>2400</v>
       </c>
       <c r="K11" s="22">
-        <v>72467</v>
+        <v>72468</v>
       </c>
       <c r="L11" s="10">
         <f t="shared" si="3"/>
-        <v>0.84079174836696102</v>
+        <v>0.84080335077562107</v>
       </c>
       <c r="M11" s="6">
         <v>247374</v>
@@ -1354,14 +1354,14 @@
       </c>
       <c r="O11" s="9">
         <f t="shared" si="4"/>
-        <v>26173</v>
+        <v>26174</v>
       </c>
       <c r="P11" s="22">
-        <v>235060</v>
+        <v>235061</v>
       </c>
       <c r="Q11" s="10">
         <f t="shared" si="5"/>
-        <v>0.95022112267255254</v>
+        <v>0.95022516513457356</v>
       </c>
       <c r="R11" s="6">
         <v>84164</v>
@@ -1371,14 +1371,14 @@
       </c>
       <c r="T11" s="9">
         <f t="shared" si="6"/>
-        <v>2723</v>
+        <v>2724</v>
       </c>
       <c r="U11" s="22">
-        <v>75304</v>
+        <v>75305</v>
       </c>
       <c r="V11" s="10">
         <f t="shared" si="7"/>
-        <v>0.89472933795922249</v>
+        <v>0.89474121952378693</v>
       </c>
       <c r="W11" s="6">
         <v>84375</v>
@@ -1388,14 +1388,14 @@
       </c>
       <c r="Y11" s="9">
         <f t="shared" si="8"/>
-        <v>3195</v>
+        <v>3196</v>
       </c>
       <c r="Z11" s="22">
-        <v>76218</v>
+        <v>76219</v>
       </c>
       <c r="AA11" s="10">
         <f t="shared" si="9"/>
-        <v>0.90332444444444449</v>
+        <v>0.9033362962962963</v>
       </c>
       <c r="AB11" s="6">
         <v>254559</v>
@@ -1405,14 +1405,14 @@
       </c>
       <c r="AD11" s="9">
         <f t="shared" si="10"/>
-        <v>28238</v>
+        <v>28240</v>
       </c>
       <c r="AE11" s="22">
-        <v>243561</v>
+        <v>243563</v>
       </c>
       <c r="AF11" s="10">
         <f t="shared" si="11"/>
-        <v>0.95679587050546244</v>
+        <v>0.95680372723022955</v>
       </c>
       <c r="AG11" s="6">
         <v>85473</v>
@@ -1439,14 +1439,14 @@
       </c>
       <c r="AN11" s="9">
         <f t="shared" si="14"/>
-        <v>4030</v>
+        <v>4031</v>
       </c>
       <c r="AO11" s="22">
-        <v>76985</v>
+        <v>76986</v>
       </c>
       <c r="AP11" s="10">
         <f t="shared" si="15"/>
-        <v>0.89415549722409349</v>
+        <v>0.89416711189574671</v>
       </c>
       <c r="AQ11" s="6">
         <v>264808</v>
@@ -1642,14 +1642,14 @@
       </c>
       <c r="E13" s="9">
         <f t="shared" si="0"/>
-        <v>16188</v>
+        <v>16193</v>
       </c>
       <c r="F13" s="22">
-        <v>75587</v>
+        <v>75592</v>
       </c>
       <c r="G13" s="10">
         <f t="shared" si="1"/>
-        <v>0.88540470891413847</v>
+        <v>0.88546327749795006</v>
       </c>
       <c r="H13" s="6">
         <v>34516</v>
@@ -1676,14 +1676,14 @@
       </c>
       <c r="O13" s="9">
         <f t="shared" si="4"/>
-        <v>21057</v>
+        <v>21060</v>
       </c>
       <c r="P13" s="22">
-        <v>87507</v>
+        <v>87510</v>
       </c>
       <c r="Q13" s="10">
         <f t="shared" si="5"/>
-        <v>0.8743879773776454</v>
+        <v>0.87441795399588318</v>
       </c>
       <c r="R13" s="6">
         <v>34094</v>
@@ -1727,14 +1727,14 @@
       </c>
       <c r="AD13" s="9">
         <f t="shared" si="10"/>
-        <v>22127</v>
+        <v>22132</v>
       </c>
       <c r="AE13" s="22">
-        <v>87324</v>
+        <v>87329</v>
       </c>
       <c r="AF13" s="10">
         <f t="shared" si="11"/>
-        <v>0.87537591723806085</v>
+        <v>0.87542603953646903</v>
       </c>
       <c r="AG13" s="6">
         <v>35615</v>
@@ -1778,14 +1778,14 @@
       </c>
       <c r="AS13" s="9">
         <f t="shared" si="16"/>
-        <v>28025</v>
+        <v>28029</v>
       </c>
       <c r="AT13" s="22">
-        <v>92874</v>
+        <v>92878</v>
       </c>
       <c r="AU13" s="10">
         <f t="shared" si="17"/>
-        <v>0.86317335216922564</v>
+        <v>0.8632105282724265</v>
       </c>
     </row>
     <row r="14" spans="1:48" x14ac:dyDescent="0.3">
@@ -1939,14 +1939,14 @@
       </c>
       <c r="AS14" s="9">
         <f t="shared" si="16"/>
-        <v>65589</v>
+        <v>65590</v>
       </c>
       <c r="AT14" s="22">
-        <v>321231</v>
+        <v>321232</v>
       </c>
       <c r="AU14" s="10">
         <f t="shared" si="17"/>
-        <v>0.93385991127442713</v>
+        <v>0.93386281840328855</v>
       </c>
     </row>
     <row r="15" spans="1:48" x14ac:dyDescent="0.3">
@@ -1964,14 +1964,14 @@
       </c>
       <c r="E15" s="9">
         <f t="shared" si="0"/>
-        <v>60326</v>
+        <v>60327</v>
       </c>
       <c r="F15" s="22">
-        <v>433309</v>
+        <v>433310</v>
       </c>
       <c r="G15" s="10">
         <f t="shared" si="1"/>
-        <v>0.97819481316934853</v>
+        <v>0.9781970706687616</v>
       </c>
       <c r="H15" s="6">
         <v>156654</v>
@@ -2100,14 +2100,14 @@
       </c>
       <c r="AS15" s="9">
         <f t="shared" si="16"/>
-        <v>100190</v>
+        <v>100191</v>
       </c>
       <c r="AT15" s="22">
-        <v>549340</v>
+        <v>549341</v>
       </c>
       <c r="AU15" s="10">
         <f t="shared" si="17"/>
-        <v>0.92735645844165493</v>
+        <v>0.92735814657006066</v>
       </c>
     </row>
     <row r="16" spans="1:48" x14ac:dyDescent="0.3">
@@ -2125,14 +2125,14 @@
       </c>
       <c r="E16" s="9">
         <f t="shared" si="0"/>
-        <v>69316</v>
+        <v>69318</v>
       </c>
       <c r="F16" s="22">
-        <v>377589</v>
+        <v>377591</v>
       </c>
       <c r="G16" s="10">
         <f t="shared" si="1"/>
-        <v>0.94509480007508917</v>
+        <v>0.94509980601964838</v>
       </c>
       <c r="H16" s="6">
         <v>126607</v>
@@ -2142,14 +2142,14 @@
       </c>
       <c r="J16" s="9">
         <f t="shared" si="2"/>
-        <v>5697</v>
+        <v>5699</v>
       </c>
       <c r="K16" s="22">
-        <v>102462</v>
+        <v>102464</v>
       </c>
       <c r="L16" s="10">
         <f t="shared" si="3"/>
-        <v>0.80929174532213854</v>
+        <v>0.80930754223700108</v>
       </c>
       <c r="M16" s="6">
         <v>435929</v>
@@ -2159,14 +2159,14 @@
       </c>
       <c r="O16" s="9">
         <f t="shared" si="4"/>
-        <v>77973</v>
+        <v>77978</v>
       </c>
       <c r="P16" s="22">
-        <v>411127</v>
+        <v>411132</v>
       </c>
       <c r="Q16" s="10">
         <f t="shared" si="5"/>
-        <v>0.94310541395502479</v>
+        <v>0.94311688371271474</v>
       </c>
       <c r="R16" s="6">
         <v>119115</v>
@@ -2176,14 +2176,14 @@
       </c>
       <c r="T16" s="9">
         <f t="shared" si="6"/>
-        <v>6367</v>
+        <v>6369</v>
       </c>
       <c r="U16" s="22">
-        <v>105082</v>
+        <v>105084</v>
       </c>
       <c r="V16" s="10">
         <f t="shared" si="7"/>
-        <v>0.88218948075389325</v>
+        <v>0.88220627125047224</v>
       </c>
       <c r="W16" s="6">
         <v>119566</v>
@@ -2193,14 +2193,14 @@
       </c>
       <c r="Y16" s="9">
         <f t="shared" si="8"/>
-        <v>7874</v>
+        <v>7876</v>
       </c>
       <c r="Z16" s="22">
-        <v>107160</v>
+        <v>107162</v>
       </c>
       <c r="AA16" s="10">
         <f t="shared" si="9"/>
-        <v>0.89624140641988526</v>
+        <v>0.89625813358312567</v>
       </c>
       <c r="AB16" s="6">
         <v>433360</v>
@@ -2210,14 +2210,14 @@
       </c>
       <c r="AD16" s="9">
         <f t="shared" si="10"/>
-        <v>79137</v>
+        <v>79140</v>
       </c>
       <c r="AE16" s="22">
-        <v>412173</v>
+        <v>412176</v>
       </c>
       <c r="AF16" s="10">
         <f t="shared" si="11"/>
-        <v>0.95110993169651104</v>
+        <v>0.95111685434742477</v>
       </c>
       <c r="AG16" s="6">
         <v>121543</v>
@@ -2227,14 +2227,14 @@
       </c>
       <c r="AI16" s="9">
         <f t="shared" si="12"/>
-        <v>8638</v>
+        <v>8641</v>
       </c>
       <c r="AJ16" s="22">
-        <v>107465</v>
+        <v>107468</v>
       </c>
       <c r="AK16" s="10">
         <f t="shared" si="13"/>
-        <v>0.88417267962778601</v>
+        <v>0.88419736225039702</v>
       </c>
       <c r="AL16" s="6">
         <v>122081</v>
@@ -2244,14 +2244,14 @@
       </c>
       <c r="AN16" s="9">
         <f t="shared" si="14"/>
-        <v>9226</v>
+        <v>9228</v>
       </c>
       <c r="AO16" s="22">
-        <v>107664</v>
+        <v>107666</v>
       </c>
       <c r="AP16" s="10">
         <f t="shared" si="15"/>
-        <v>0.88190627534178123</v>
+        <v>0.88192265790745483</v>
       </c>
       <c r="AQ16" s="6">
         <v>455889</v>
@@ -2261,14 +2261,14 @@
       </c>
       <c r="AS16" s="9">
         <f t="shared" si="16"/>
-        <v>94220</v>
+        <v>94223</v>
       </c>
       <c r="AT16" s="22">
-        <v>430115</v>
+        <v>430118</v>
       </c>
       <c r="AU16" s="10">
         <f t="shared" si="17"/>
-        <v>0.94346430819782889</v>
+        <v>0.94347088874704155</v>
       </c>
     </row>
     <row r="17" spans="1:47" x14ac:dyDescent="0.3">
@@ -2286,14 +2286,14 @@
       </c>
       <c r="E17" s="9">
         <f t="shared" si="0"/>
-        <v>125742</v>
+        <v>125743</v>
       </c>
       <c r="F17" s="22">
-        <v>680420</v>
+        <v>680421</v>
       </c>
       <c r="G17" s="10">
         <f t="shared" si="1"/>
-        <v>0.92197082408544107</v>
+        <v>0.92197217908797491</v>
       </c>
       <c r="H17" s="6">
         <v>278909</v>
@@ -2320,14 +2320,14 @@
       </c>
       <c r="O17" s="9">
         <f t="shared" si="4"/>
-        <v>168604</v>
+        <v>168606</v>
       </c>
       <c r="P17" s="22">
-        <v>800812</v>
+        <v>800814</v>
       </c>
       <c r="Q17" s="10">
         <f t="shared" si="5"/>
-        <v>0.90196157935521071</v>
+        <v>0.90196383197275232</v>
       </c>
       <c r="R17" s="6">
         <v>272330</v>
@@ -2337,14 +2337,14 @@
       </c>
       <c r="T17" s="9">
         <f t="shared" si="6"/>
-        <v>23000</v>
+        <v>23001</v>
       </c>
       <c r="U17" s="22">
-        <v>228339</v>
+        <v>228340</v>
       </c>
       <c r="V17" s="10">
         <f t="shared" si="7"/>
-        <v>0.83846436308889949</v>
+        <v>0.83846803510446888</v>
       </c>
       <c r="W17" s="6">
         <v>275780</v>
@@ -2354,14 +2354,14 @@
       </c>
       <c r="Y17" s="9">
         <f t="shared" si="8"/>
-        <v>28165</v>
+        <v>28166</v>
       </c>
       <c r="Z17" s="22">
-        <v>235985</v>
+        <v>235986</v>
       </c>
       <c r="AA17" s="10">
         <f t="shared" si="9"/>
-        <v>0.85570019580825296</v>
+        <v>0.85570382188701144</v>
       </c>
       <c r="AB17" s="6">
         <v>847512</v>
@@ -2371,14 +2371,14 @@
       </c>
       <c r="AD17" s="9">
         <f t="shared" si="10"/>
-        <v>170077</v>
+        <v>170080</v>
       </c>
       <c r="AE17" s="22">
-        <v>769906</v>
+        <v>769909</v>
       </c>
       <c r="AF17" s="10">
         <f t="shared" si="11"/>
-        <v>0.90843079508018765</v>
+        <v>0.90843433485307579</v>
       </c>
       <c r="AG17" s="6">
         <v>284469</v>
@@ -2422,14 +2422,14 @@
       </c>
       <c r="AS17" s="9">
         <f t="shared" si="16"/>
-        <v>211263</v>
+        <v>211266</v>
       </c>
       <c r="AT17" s="22">
-        <v>816216</v>
+        <v>816219</v>
       </c>
       <c r="AU17" s="10">
         <f t="shared" si="17"/>
-        <v>0.89383776538368453</v>
+        <v>0.8938410506823018</v>
       </c>
     </row>
     <row r="18" spans="1:47" x14ac:dyDescent="0.3">
@@ -2583,14 +2583,14 @@
       </c>
       <c r="AS18" s="9">
         <f t="shared" si="16"/>
-        <v>69316</v>
+        <v>69317</v>
       </c>
       <c r="AT18" s="22">
-        <v>200041</v>
+        <v>200042</v>
       </c>
       <c r="AU18" s="10">
         <f t="shared" si="17"/>
-        <v>0.83789964857313992</v>
+        <v>0.83790383721271167</v>
       </c>
     </row>
     <row r="19" spans="1:47" x14ac:dyDescent="0.3">
@@ -2930,14 +2930,14 @@
       </c>
       <c r="E21" s="9">
         <f t="shared" si="0"/>
-        <v>834</v>
+        <v>836</v>
       </c>
       <c r="F21" s="22">
-        <v>3135</v>
+        <v>3137</v>
       </c>
       <c r="G21" s="10">
         <f t="shared" si="1"/>
-        <v>0.8003574163900945</v>
+        <v>0.8008680112330866</v>
       </c>
       <c r="H21" s="6">
         <v>3140</v>
@@ -3210,14 +3210,14 @@
       </c>
       <c r="AN22" s="9">
         <f t="shared" si="14"/>
-        <v>872</v>
+        <v>873</v>
       </c>
       <c r="AO22" s="22">
-        <v>3108</v>
+        <v>3109</v>
       </c>
       <c r="AP22" s="10">
         <f t="shared" si="15"/>
-        <v>0.62914979757085021</v>
+        <v>0.62935222672064772</v>
       </c>
       <c r="AQ22" s="6">
         <v>8603</v>
@@ -3227,14 +3227,14 @@
       </c>
       <c r="AS22" s="9">
         <f t="shared" si="16"/>
-        <v>2112</v>
+        <v>2113</v>
       </c>
       <c r="AT22" s="22">
-        <v>6013</v>
+        <v>6014</v>
       </c>
       <c r="AU22" s="10">
         <f t="shared" si="17"/>
-        <v>0.6989422294548413</v>
+        <v>0.69905846797628735</v>
       </c>
     </row>
     <row r="23" spans="1:47" x14ac:dyDescent="0.3">
@@ -3498,14 +3498,14 @@
       </c>
       <c r="AD24" s="9">
         <f t="shared" si="10"/>
-        <v>3433</v>
+        <v>3434</v>
       </c>
       <c r="AE24" s="22">
-        <v>14732</v>
+        <v>14733</v>
       </c>
       <c r="AF24" s="10">
         <f t="shared" si="11"/>
-        <v>0.87357685009487662</v>
+        <v>0.87363614800759015</v>
       </c>
       <c r="AG24" s="6">
         <v>7129</v>
@@ -3769,14 +3769,14 @@
       </c>
       <c r="O26" s="9">
         <f t="shared" si="4"/>
-        <v>26357</v>
+        <v>26358</v>
       </c>
       <c r="P26" s="22">
-        <v>90686</v>
+        <v>90687</v>
       </c>
       <c r="Q26" s="10">
         <f t="shared" si="5"/>
-        <v>0.7933269764064701</v>
+        <v>0.79333572447096079</v>
       </c>
       <c r="R26" s="6">
         <v>54732</v>
@@ -3786,14 +3786,14 @@
       </c>
       <c r="T26" s="9">
         <f t="shared" si="6"/>
-        <v>7816</v>
+        <v>7817</v>
       </c>
       <c r="U26" s="22">
-        <v>38326</v>
+        <v>38327</v>
       </c>
       <c r="V26" s="10">
         <f t="shared" si="7"/>
-        <v>0.70024848351969593</v>
+        <v>0.70026675436673247</v>
       </c>
       <c r="W26" s="6">
         <v>55786</v>
@@ -3803,14 +3803,14 @@
       </c>
       <c r="Y26" s="9">
         <f t="shared" si="8"/>
-        <v>8881</v>
+        <v>8882</v>
       </c>
       <c r="Z26" s="22">
-        <v>39490</v>
+        <v>39491</v>
       </c>
       <c r="AA26" s="10">
         <f t="shared" si="9"/>
-        <v>0.70788369841895815</v>
+        <v>0.70790162406338508</v>
       </c>
       <c r="AB26" s="6">
         <v>114563</v>
@@ -3820,14 +3820,14 @@
       </c>
       <c r="AD26" s="9">
         <f t="shared" si="10"/>
-        <v>28766</v>
+        <v>28767</v>
       </c>
       <c r="AE26" s="22">
-        <v>91594</v>
+        <v>91595</v>
       </c>
       <c r="AF26" s="10">
         <f t="shared" si="11"/>
-        <v>0.7995076944563253</v>
+        <v>0.79951642327802175</v>
       </c>
       <c r="AG26" s="6">
         <v>56208</v>
@@ -3837,14 +3837,14 @@
       </c>
       <c r="AI26" s="9">
         <f t="shared" si="12"/>
-        <v>10040</v>
+        <v>10041</v>
       </c>
       <c r="AJ26" s="22">
-        <v>39517</v>
+        <v>39518</v>
       </c>
       <c r="AK26" s="10">
         <f t="shared" si="13"/>
-        <v>0.70304938798747507</v>
+        <v>0.70306717904924565</v>
       </c>
       <c r="AL26" s="6">
         <v>57763</v>
@@ -3854,14 +3854,14 @@
       </c>
       <c r="AN26" s="9">
         <f t="shared" si="14"/>
-        <v>10831</v>
+        <v>10832</v>
       </c>
       <c r="AO26" s="22">
-        <v>39843</v>
+        <v>39844</v>
       </c>
       <c r="AP26" s="10">
         <f t="shared" si="15"/>
-        <v>0.68976680574069904</v>
+        <v>0.68978411786091443</v>
       </c>
       <c r="AQ26" s="6">
         <v>122022</v>
@@ -3871,14 +3871,14 @@
       </c>
       <c r="AS26" s="9">
         <f t="shared" si="16"/>
-        <v>35929</v>
+        <v>35930</v>
       </c>
       <c r="AT26" s="22">
-        <v>95615</v>
+        <v>95616</v>
       </c>
       <c r="AU26" s="10">
         <f t="shared" si="17"/>
-        <v>0.78358820540558261</v>
+        <v>0.78359640064906333</v>
       </c>
     </row>
     <row r="27" spans="1:47" x14ac:dyDescent="0.3">
@@ -3896,14 +3896,14 @@
       </c>
       <c r="E27" s="9">
         <f t="shared" si="0"/>
-        <v>27880</v>
+        <v>27882</v>
       </c>
       <c r="F27" s="22">
-        <v>311090</v>
+        <v>311092</v>
       </c>
       <c r="G27" s="10">
         <f t="shared" si="1"/>
-        <v>0.89646129906057292</v>
+        <v>0.89646706241715179</v>
       </c>
       <c r="H27" s="6">
         <v>162480</v>
@@ -3930,14 +3930,14 @@
       </c>
       <c r="O27" s="9">
         <f t="shared" si="4"/>
-        <v>50597</v>
+        <v>50598</v>
       </c>
       <c r="P27" s="22">
-        <v>384725</v>
+        <v>384726</v>
       </c>
       <c r="Q27" s="10">
         <f t="shared" si="5"/>
-        <v>0.92475079982020569</v>
+        <v>0.92475320348724011</v>
       </c>
       <c r="R27" s="6">
         <v>158774</v>
@@ -3947,14 +3947,14 @@
       </c>
       <c r="T27" s="9">
         <f t="shared" si="6"/>
-        <v>14617</v>
+        <v>14618</v>
       </c>
       <c r="U27" s="22">
-        <v>136500</v>
+        <v>136501</v>
       </c>
       <c r="V27" s="10">
         <f t="shared" si="7"/>
-        <v>0.85971254739440961</v>
+        <v>0.85971884565483014</v>
       </c>
       <c r="W27" s="6">
         <v>161708</v>
@@ -3964,14 +3964,14 @@
       </c>
       <c r="Y27" s="9">
         <f t="shared" si="8"/>
-        <v>16785</v>
+        <v>16787</v>
       </c>
       <c r="Z27" s="22">
-        <v>140071</v>
+        <v>140073</v>
       </c>
       <c r="AA27" s="10">
         <f t="shared" si="9"/>
-        <v>0.8661970960001979</v>
+        <v>0.86620946397209786</v>
       </c>
       <c r="AB27" s="6">
         <v>443892</v>
@@ -3981,14 +3981,14 @@
       </c>
       <c r="AD27" s="9">
         <f t="shared" si="10"/>
-        <v>64100</v>
+        <v>64102</v>
       </c>
       <c r="AE27" s="22">
-        <v>408368</v>
+        <v>408370</v>
       </c>
       <c r="AF27" s="10">
         <f t="shared" si="11"/>
-        <v>0.91997152460508413</v>
+        <v>0.91997603020554553</v>
       </c>
       <c r="AG27" s="6">
         <v>164959</v>
@@ -3998,14 +3998,14 @@
       </c>
       <c r="AI27" s="9">
         <f t="shared" si="12"/>
-        <v>19961</v>
+        <v>19962</v>
       </c>
       <c r="AJ27" s="22">
-        <v>141795</v>
+        <v>141796</v>
       </c>
       <c r="AK27" s="10">
         <f t="shared" si="13"/>
-        <v>0.85957722828096683</v>
+        <v>0.85958329039337045</v>
       </c>
       <c r="AL27" s="6">
         <v>167478</v>
@@ -4015,14 +4015,14 @@
       </c>
       <c r="AN27" s="9">
         <f t="shared" si="14"/>
-        <v>22153</v>
+        <v>22155</v>
       </c>
       <c r="AO27" s="22">
-        <v>143256</v>
+        <v>143258</v>
       </c>
       <c r="AP27" s="10">
         <f t="shared" si="15"/>
-        <v>0.85537204886611973</v>
+        <v>0.85538399073311122</v>
       </c>
       <c r="AQ27" s="6">
         <v>472982</v>
@@ -4032,14 +4032,14 @@
       </c>
       <c r="AS27" s="9">
         <f t="shared" si="16"/>
-        <v>87042</v>
+        <v>87044</v>
       </c>
       <c r="AT27" s="22">
-        <v>430563</v>
+        <v>430565</v>
       </c>
       <c r="AU27" s="10">
         <f t="shared" si="17"/>
-        <v>0.9103158259722357</v>
+        <v>0.91032005446296049</v>
       </c>
     </row>
     <row r="28" spans="1:47" x14ac:dyDescent="0.3">
@@ -4193,14 +4193,14 @@
       </c>
       <c r="AS28" s="9">
         <f t="shared" si="16"/>
-        <v>29724</v>
+        <v>29725</v>
       </c>
       <c r="AT28" s="22">
-        <v>103464</v>
+        <v>103465</v>
       </c>
       <c r="AU28" s="10">
         <f t="shared" si="17"/>
-        <v>0.88267060238702577</v>
+        <v>0.88267913357277528</v>
       </c>
     </row>
     <row r="29" spans="1:47" x14ac:dyDescent="0.3">
@@ -4218,14 +4218,14 @@
       </c>
       <c r="E29" s="9">
         <f t="shared" si="0"/>
-        <v>25968</v>
+        <v>25970</v>
       </c>
       <c r="F29" s="22">
-        <v>122774</v>
+        <v>122776</v>
       </c>
       <c r="G29" s="10">
         <f t="shared" si="1"/>
-        <v>0.87774084003574615</v>
+        <v>0.87775513851653264</v>
       </c>
       <c r="H29" s="6">
         <v>57678</v>
@@ -4235,14 +4235,14 @@
       </c>
       <c r="J29" s="9">
         <f t="shared" si="2"/>
-        <v>6662</v>
+        <v>6664</v>
       </c>
       <c r="K29" s="22">
-        <v>43285</v>
+        <v>43287</v>
       </c>
       <c r="L29" s="10">
         <f t="shared" si="3"/>
-        <v>0.7504594472762578</v>
+        <v>0.75049412254239056</v>
       </c>
       <c r="M29" s="6">
         <v>162133</v>
@@ -4252,14 +4252,14 @@
       </c>
       <c r="O29" s="9">
         <f t="shared" si="4"/>
-        <v>34785</v>
+        <v>34789</v>
       </c>
       <c r="P29" s="22">
-        <v>139303</v>
+        <v>139307</v>
       </c>
       <c r="Q29" s="10">
         <f t="shared" si="5"/>
-        <v>0.85918967761035692</v>
+        <v>0.85921434871371039</v>
       </c>
       <c r="R29" s="6">
         <v>59901</v>
@@ -4269,14 +4269,14 @@
       </c>
       <c r="T29" s="9">
         <f t="shared" si="6"/>
-        <v>7654</v>
+        <v>7656</v>
       </c>
       <c r="U29" s="22">
-        <v>45112</v>
+        <v>45114</v>
       </c>
       <c r="V29" s="10">
         <f t="shared" si="7"/>
-        <v>0.7531092970067278</v>
+        <v>0.75314268543096108</v>
       </c>
       <c r="W29" s="6">
         <v>61437</v>
@@ -4286,14 +4286,14 @@
       </c>
       <c r="Y29" s="9">
         <f t="shared" si="8"/>
-        <v>8529</v>
+        <v>8531</v>
       </c>
       <c r="Z29" s="22">
-        <v>46432</v>
+        <v>46434</v>
       </c>
       <c r="AA29" s="10">
         <f t="shared" si="9"/>
-        <v>0.75576606930676948</v>
+        <v>0.75579862297963762</v>
       </c>
       <c r="AB29" s="6">
         <v>168723</v>
@@ -4303,14 +4303,14 @@
       </c>
       <c r="AD29" s="9">
         <f t="shared" si="10"/>
-        <v>39107</v>
+        <v>39110</v>
       </c>
       <c r="AE29" s="22">
-        <v>143308</v>
+        <v>143311</v>
       </c>
       <c r="AF29" s="10">
         <f t="shared" si="11"/>
-        <v>0.84936849155124083</v>
+        <v>0.84938627217391816</v>
       </c>
       <c r="AG29" s="6">
         <v>64080</v>
@@ -4320,14 +4320,14 @@
       </c>
       <c r="AI29" s="9">
         <f t="shared" si="12"/>
-        <v>9941</v>
+        <v>9943</v>
       </c>
       <c r="AJ29" s="22">
-        <v>47206</v>
+        <v>47208</v>
       </c>
       <c r="AK29" s="10">
         <f t="shared" si="13"/>
-        <v>0.73667290886392012</v>
+        <v>0.73670411985018724</v>
       </c>
       <c r="AL29" s="6">
         <v>65194</v>
@@ -4337,14 +4337,14 @@
       </c>
       <c r="AN29" s="9">
         <f t="shared" si="14"/>
-        <v>10804</v>
+        <v>10807</v>
       </c>
       <c r="AO29" s="22">
-        <v>47726</v>
+        <v>47729</v>
       </c>
       <c r="AP29" s="10">
         <f t="shared" si="15"/>
-        <v>0.73206123262876954</v>
+        <v>0.73210724913335579</v>
       </c>
       <c r="AQ29" s="6">
         <v>183516</v>
@@ -4354,14 +4354,14 @@
       </c>
       <c r="AS29" s="9">
         <f t="shared" si="16"/>
-        <v>50061</v>
+        <v>50066</v>
       </c>
       <c r="AT29" s="22">
-        <v>152145</v>
+        <v>152150</v>
       </c>
       <c r="AU29" s="10">
         <f t="shared" si="17"/>
-        <v>0.82905577715294576</v>
+        <v>0.82908302273371259</v>
       </c>
     </row>
     <row r="30" spans="1:47" x14ac:dyDescent="0.3">
@@ -4379,14 +4379,14 @@
       </c>
       <c r="E30" s="9">
         <f t="shared" si="0"/>
-        <v>16365</v>
+        <v>16367</v>
       </c>
       <c r="F30" s="22">
-        <v>72627</v>
+        <v>72629</v>
       </c>
       <c r="G30" s="10">
         <f t="shared" si="1"/>
-        <v>0.8708377798294944</v>
+        <v>0.87086176093238532</v>
       </c>
       <c r="H30" s="6">
         <v>37862</v>
@@ -4396,14 +4396,14 @@
       </c>
       <c r="J30" s="9">
         <f t="shared" si="2"/>
-        <v>3852</v>
+        <v>3854</v>
       </c>
       <c r="K30" s="22">
-        <v>29247</v>
+        <v>29249</v>
       </c>
       <c r="L30" s="10">
         <f t="shared" si="3"/>
-        <v>0.7724631556705932</v>
+        <v>0.77251597908192915</v>
       </c>
       <c r="M30" s="6">
         <v>93983</v>
@@ -4430,14 +4430,14 @@
       </c>
       <c r="T30" s="9">
         <f t="shared" si="6"/>
-        <v>4430</v>
+        <v>4431</v>
       </c>
       <c r="U30" s="22">
-        <v>30026</v>
+        <v>30027</v>
       </c>
       <c r="V30" s="10">
         <f t="shared" si="7"/>
-        <v>0.81734538327526129</v>
+        <v>0.81737260452961669</v>
       </c>
       <c r="W30" s="6">
         <v>37342</v>
@@ -4447,14 +4447,14 @@
       </c>
       <c r="Y30" s="9">
         <f t="shared" si="8"/>
-        <v>5035</v>
+        <v>5036</v>
       </c>
       <c r="Z30" s="22">
-        <v>30690</v>
+        <v>30691</v>
       </c>
       <c r="AA30" s="10">
         <f t="shared" si="9"/>
-        <v>0.82186278185421247</v>
+        <v>0.821889561351829</v>
       </c>
       <c r="AB30" s="6">
         <v>90937</v>
@@ -4464,14 +4464,14 @@
       </c>
       <c r="AD30" s="9">
         <f t="shared" si="10"/>
-        <v>21955</v>
+        <v>21958</v>
       </c>
       <c r="AE30" s="22">
-        <v>79607</v>
+        <v>79610</v>
       </c>
       <c r="AF30" s="10">
         <f t="shared" si="11"/>
-        <v>0.87540824966735209</v>
+        <v>0.8754412395394614</v>
       </c>
       <c r="AG30" s="6">
         <v>37890</v>
@@ -4481,14 +4481,14 @@
       </c>
       <c r="AI30" s="9">
         <f t="shared" si="12"/>
-        <v>5936</v>
+        <v>5937</v>
       </c>
       <c r="AJ30" s="22">
-        <v>30639</v>
+        <v>30640</v>
       </c>
       <c r="AK30" s="10">
         <f t="shared" si="13"/>
-        <v>0.80863024544734763</v>
+        <v>0.80865663763525997</v>
       </c>
       <c r="AL30" s="6">
         <v>37957</v>
@@ -4498,14 +4498,14 @@
       </c>
       <c r="AN30" s="9">
         <f t="shared" si="14"/>
-        <v>6520</v>
+        <v>6521</v>
       </c>
       <c r="AO30" s="22">
-        <v>30730</v>
+        <v>30731</v>
       </c>
       <c r="AP30" s="10">
         <f t="shared" si="15"/>
-        <v>0.80960033722370051</v>
+        <v>0.80962668282530237</v>
       </c>
       <c r="AQ30" s="6">
         <v>94349</v>
@@ -4515,14 +4515,14 @@
       </c>
       <c r="AS30" s="9">
         <f t="shared" si="16"/>
-        <v>27512</v>
+        <v>27514</v>
       </c>
       <c r="AT30" s="22">
-        <v>81678</v>
+        <v>81680</v>
       </c>
       <c r="AU30" s="10">
         <f t="shared" si="17"/>
-        <v>0.86570074934551511</v>
+        <v>0.86572194723844453</v>
       </c>
     </row>
     <row r="31" spans="1:47" x14ac:dyDescent="0.3">
@@ -4540,14 +4540,14 @@
       </c>
       <c r="E31" s="9">
         <f t="shared" si="0"/>
-        <v>43648</v>
+        <v>43650</v>
       </c>
       <c r="F31" s="22">
-        <v>240840</v>
+        <v>240842</v>
       </c>
       <c r="G31" s="10">
         <f t="shared" si="1"/>
-        <v>0.9359988807188272</v>
+        <v>0.93600665350474921</v>
       </c>
       <c r="H31" s="6">
         <v>94897</v>
@@ -4676,14 +4676,14 @@
       </c>
       <c r="AS31" s="9">
         <f t="shared" si="16"/>
-        <v>72143</v>
+        <v>72145</v>
       </c>
       <c r="AT31" s="22">
-        <v>273901</v>
+        <v>273903</v>
       </c>
       <c r="AU31" s="10">
         <f t="shared" si="17"/>
-        <v>0.89824516526798037</v>
+        <v>0.89825172417185639</v>
       </c>
     </row>
     <row r="32" spans="1:47" x14ac:dyDescent="0.3">
@@ -4701,14 +4701,14 @@
       </c>
       <c r="E32" s="9">
         <f t="shared" si="0"/>
-        <v>68649</v>
+        <v>68658</v>
       </c>
       <c r="F32" s="22">
-        <v>540571</v>
+        <v>540580</v>
       </c>
       <c r="G32" s="10">
         <f t="shared" si="1"/>
-        <v>0.95754412006964973</v>
+        <v>0.95756006228090529</v>
       </c>
       <c r="H32" s="6">
         <v>224696</v>
@@ -4718,14 +4718,14 @@
       </c>
       <c r="J32" s="9">
         <f t="shared" si="2"/>
-        <v>8453</v>
+        <v>8455</v>
       </c>
       <c r="K32" s="22">
-        <v>204573</v>
+        <v>204575</v>
       </c>
       <c r="L32" s="10">
         <f t="shared" si="3"/>
-        <v>0.9104434435860006</v>
+        <v>0.91045234450101475</v>
       </c>
       <c r="M32" s="6">
         <v>682019</v>
@@ -4735,14 +4735,14 @@
       </c>
       <c r="O32" s="9">
         <f t="shared" si="4"/>
-        <v>94821</v>
+        <v>94826</v>
       </c>
       <c r="P32" s="22">
-        <v>656090</v>
+        <v>656095</v>
       </c>
       <c r="Q32" s="10">
         <f t="shared" si="5"/>
-        <v>0.96198199756898273</v>
+        <v>0.96198932874304088</v>
       </c>
       <c r="R32" s="6">
         <v>225967</v>
@@ -4752,14 +4752,14 @@
       </c>
       <c r="T32" s="9">
         <f t="shared" si="6"/>
-        <v>9813</v>
+        <v>9814</v>
       </c>
       <c r="U32" s="22">
-        <v>212616</v>
+        <v>212617</v>
       </c>
       <c r="V32" s="10">
         <f t="shared" si="7"/>
-        <v>0.94091615147344521</v>
+        <v>0.9409205768983967</v>
       </c>
       <c r="W32" s="6">
         <v>228262</v>
@@ -4769,14 +4769,14 @@
       </c>
       <c r="Y32" s="9">
         <f t="shared" si="8"/>
-        <v>11704</v>
+        <v>11705</v>
       </c>
       <c r="Z32" s="22">
-        <v>216309</v>
+        <v>216310</v>
       </c>
       <c r="AA32" s="10">
         <f t="shared" si="9"/>
-        <v>0.94763473552321453</v>
+        <v>0.94763911645389942</v>
       </c>
       <c r="AB32" s="6">
         <v>698869</v>
@@ -4786,14 +4786,14 @@
       </c>
       <c r="AD32" s="9">
         <f t="shared" si="10"/>
-        <v>100361</v>
+        <v>100363</v>
       </c>
       <c r="AE32" s="22">
-        <v>678195</v>
+        <v>678197</v>
       </c>
       <c r="AF32" s="10">
         <f t="shared" si="11"/>
-        <v>0.97041791809337663</v>
+        <v>0.97042077986003095</v>
       </c>
       <c r="AG32" s="6">
         <v>232401</v>
@@ -4803,14 +4803,14 @@
       </c>
       <c r="AI32" s="9">
         <f t="shared" si="12"/>
-        <v>13766</v>
+        <v>13767</v>
       </c>
       <c r="AJ32" s="22">
-        <v>218605</v>
+        <v>218606</v>
       </c>
       <c r="AK32" s="10">
         <f t="shared" si="13"/>
-        <v>0.94063708848068639</v>
+        <v>0.94064139138816094</v>
       </c>
       <c r="AL32" s="6">
         <v>234200</v>
@@ -4820,14 +4820,14 @@
       </c>
       <c r="AN32" s="9">
         <f t="shared" si="14"/>
-        <v>14850</v>
+        <v>14852</v>
       </c>
       <c r="AO32" s="22">
-        <v>219618</v>
+        <v>219620</v>
       </c>
       <c r="AP32" s="10">
         <f t="shared" si="15"/>
-        <v>0.93773697694278391</v>
+        <v>0.93774551665243377</v>
       </c>
       <c r="AQ32" s="6">
         <v>733311</v>
@@ -4837,14 +4837,14 @@
       </c>
       <c r="AS32" s="9">
         <f t="shared" si="16"/>
-        <v>118429</v>
+        <v>118431</v>
       </c>
       <c r="AT32" s="22">
-        <v>708213</v>
+        <v>708215</v>
       </c>
       <c r="AU32" s="10">
         <f t="shared" si="17"/>
-        <v>0.96577441222073579</v>
+        <v>0.96577713957652345</v>
       </c>
     </row>
     <row r="33" spans="1:47" x14ac:dyDescent="0.3">
@@ -5184,14 +5184,14 @@
       </c>
       <c r="E35" s="9">
         <f t="shared" si="0"/>
-        <v>145157</v>
+        <v>145164</v>
       </c>
       <c r="F35" s="22">
-        <v>864293</v>
+        <v>864300</v>
       </c>
       <c r="G35" s="10">
         <f t="shared" si="1"/>
-        <v>0.94469401852896295</v>
+        <v>0.94470166970527669</v>
       </c>
       <c r="H35" s="6">
         <v>336894</v>
@@ -5201,14 +5201,14 @@
       </c>
       <c r="J35" s="9">
         <f t="shared" si="2"/>
-        <v>22984</v>
+        <v>22986</v>
       </c>
       <c r="K35" s="22">
-        <v>297053</v>
+        <v>297055</v>
       </c>
       <c r="L35" s="10">
         <f t="shared" si="3"/>
-        <v>0.88174025064263539</v>
+        <v>0.88174618722803022</v>
       </c>
       <c r="M35" s="6">
         <v>1060520</v>
@@ -5218,14 +5218,14 @@
       </c>
       <c r="O35" s="9">
         <f t="shared" si="4"/>
-        <v>190488</v>
+        <v>190490</v>
       </c>
       <c r="P35" s="22">
-        <v>1004071</v>
+        <v>1004073</v>
       </c>
       <c r="Q35" s="10">
         <f t="shared" si="5"/>
-        <v>0.94677233809829142</v>
+        <v>0.94677422396560174</v>
       </c>
       <c r="R35" s="6">
         <v>338572</v>
@@ -5235,14 +5235,14 @@
       </c>
       <c r="T35" s="9">
         <f t="shared" si="6"/>
-        <v>26619</v>
+        <v>26622</v>
       </c>
       <c r="U35" s="22">
-        <v>308479</v>
+        <v>308482</v>
       </c>
       <c r="V35" s="10">
         <f t="shared" si="7"/>
-        <v>0.91111787153101853</v>
+        <v>0.91112673227555729</v>
       </c>
       <c r="W35" s="6">
         <v>341709</v>
@@ -5252,14 +5252,14 @@
       </c>
       <c r="Y35" s="9">
         <f t="shared" si="8"/>
-        <v>30169</v>
+        <v>30173</v>
       </c>
       <c r="Z35" s="22">
-        <v>313376</v>
+        <v>313380</v>
       </c>
       <c r="AA35" s="10">
         <f t="shared" si="9"/>
-        <v>0.91708441978408528</v>
+        <v>0.91709612565077303</v>
       </c>
       <c r="AB35" s="6">
         <v>1094504</v>
@@ -5269,14 +5269,14 @@
       </c>
       <c r="AD35" s="9">
         <f t="shared" si="10"/>
-        <v>211142</v>
+        <v>211149</v>
       </c>
       <c r="AE35" s="22">
-        <v>1042451</v>
+        <v>1042458</v>
       </c>
       <c r="AF35" s="10">
         <f t="shared" si="11"/>
-        <v>0.95244147120522171</v>
+        <v>0.95244786679628402</v>
       </c>
       <c r="AG35" s="6">
         <v>348478</v>
@@ -5286,14 +5286,14 @@
       </c>
       <c r="AI35" s="9">
         <f t="shared" si="12"/>
-        <v>36072</v>
+        <v>36074</v>
       </c>
       <c r="AJ35" s="22">
-        <v>316476</v>
+        <v>316478</v>
       </c>
       <c r="AK35" s="10">
         <f t="shared" si="13"/>
-        <v>0.90816636918255955</v>
+        <v>0.908172108425783</v>
       </c>
       <c r="AL35" s="6">
         <v>352081</v>
@@ -5303,14 +5303,14 @@
       </c>
       <c r="AN35" s="9">
         <f t="shared" si="14"/>
-        <v>39181</v>
+        <v>39183</v>
       </c>
       <c r="AO35" s="22">
-        <v>318221</v>
+        <v>318223</v>
       </c>
       <c r="AP35" s="10">
         <f t="shared" si="15"/>
-        <v>0.90382894845220274</v>
+        <v>0.90383462896322153</v>
       </c>
       <c r="AQ35" s="6">
         <v>1148243</v>
@@ -5320,14 +5320,14 @@
       </c>
       <c r="AS35" s="9">
         <f t="shared" si="16"/>
-        <v>254029</v>
+        <v>254038</v>
       </c>
       <c r="AT35" s="22">
-        <v>1087088</v>
+        <v>1087097</v>
       </c>
       <c r="AU35" s="10">
         <f t="shared" si="17"/>
-        <v>0.94674036767478664</v>
+        <v>0.94674820573693896</v>
       </c>
     </row>
     <row r="36" spans="1:47" x14ac:dyDescent="0.3">
@@ -5345,14 +5345,14 @@
       </c>
       <c r="E36" s="9">
         <f t="shared" si="0"/>
-        <v>76398</v>
+        <v>76405</v>
       </c>
       <c r="F36" s="22">
-        <v>460717</v>
+        <v>460724</v>
       </c>
       <c r="G36" s="10">
         <f t="shared" si="1"/>
-        <v>0.91519784190525755</v>
+        <v>0.91521174715488662</v>
       </c>
       <c r="H36" s="6">
         <v>312358</v>
@@ -5362,14 +5362,14 @@
       </c>
       <c r="J36" s="9">
         <f t="shared" si="2"/>
-        <v>32454</v>
+        <v>32461</v>
       </c>
       <c r="K36" s="22">
-        <v>276697</v>
+        <v>276704</v>
       </c>
       <c r="L36" s="10">
         <f t="shared" si="3"/>
-        <v>0.88583292247997492</v>
+        <v>0.88585533266316219</v>
       </c>
       <c r="M36" s="6">
         <v>553919</v>
@@ -5379,14 +5379,14 @@
       </c>
       <c r="O36" s="9">
         <f t="shared" si="4"/>
-        <v>94046</v>
+        <v>94053</v>
       </c>
       <c r="P36" s="22">
-        <v>494786</v>
+        <v>494793</v>
       </c>
       <c r="Q36" s="10">
         <f t="shared" si="5"/>
-        <v>0.89324612443335583</v>
+        <v>0.89325876166009832</v>
       </c>
       <c r="R36" s="6">
         <v>318679</v>
@@ -5396,14 +5396,14 @@
       </c>
       <c r="T36" s="9">
         <f t="shared" si="6"/>
-        <v>35603</v>
+        <v>35610</v>
       </c>
       <c r="U36" s="22">
-        <v>284058</v>
+        <v>284065</v>
       </c>
       <c r="V36" s="10">
         <f t="shared" si="7"/>
-        <v>0.89136089921205974</v>
+        <v>0.89138286488912044</v>
       </c>
       <c r="W36" s="6">
         <v>324721</v>
@@ -5413,14 +5413,14 @@
       </c>
       <c r="Y36" s="9">
         <f t="shared" si="8"/>
-        <v>38946</v>
+        <v>38954</v>
       </c>
       <c r="Z36" s="22">
-        <v>289562</v>
+        <v>289570</v>
       </c>
       <c r="AA36" s="10">
         <f t="shared" si="9"/>
-        <v>0.89172551205496409</v>
+        <v>0.89175014858909651</v>
       </c>
       <c r="AB36" s="6">
         <v>556414</v>
@@ -5430,14 +5430,14 @@
       </c>
       <c r="AD36" s="9">
         <f t="shared" si="10"/>
-        <v>102217</v>
+        <v>102224</v>
       </c>
       <c r="AE36" s="22">
-        <v>499744</v>
+        <v>499751</v>
       </c>
       <c r="AF36" s="10">
         <f t="shared" si="11"/>
-        <v>0.898151376493043</v>
+        <v>0.89816395705356089</v>
       </c>
       <c r="AG36" s="6">
         <v>333690</v>
@@ -5447,14 +5447,14 @@
       </c>
       <c r="AI36" s="9">
         <f t="shared" si="12"/>
-        <v>47415</v>
+        <v>47419</v>
       </c>
       <c r="AJ36" s="22">
-        <v>293774</v>
+        <v>293778</v>
       </c>
       <c r="AK36" s="10">
         <f t="shared" si="13"/>
-        <v>0.88037999340705442</v>
+        <v>0.88039198058077861</v>
       </c>
       <c r="AL36" s="6">
         <v>339216</v>
@@ -5464,14 +5464,14 @@
       </c>
       <c r="AN36" s="9">
         <f t="shared" si="14"/>
-        <v>52328</v>
+        <v>52331</v>
       </c>
       <c r="AO36" s="22">
-        <v>296764</v>
+        <v>296767</v>
       </c>
       <c r="AP36" s="10">
         <f t="shared" si="15"/>
-        <v>0.87485260129239184</v>
+        <v>0.87486144521484832</v>
       </c>
       <c r="AQ36" s="6">
         <v>590015</v>
@@ -5481,14 +5481,14 @@
       </c>
       <c r="AS36" s="9">
         <f t="shared" si="16"/>
-        <v>131189</v>
+        <v>131196</v>
       </c>
       <c r="AT36" s="22">
-        <v>521171</v>
+        <v>521178</v>
       </c>
       <c r="AU36" s="10">
         <f t="shared" si="17"/>
-        <v>0.88331822072320199</v>
+        <v>0.88333008482835185</v>
       </c>
     </row>
     <row r="37" spans="1:47" x14ac:dyDescent="0.3">
@@ -5506,14 +5506,14 @@
       </c>
       <c r="E37" s="9">
         <f t="shared" si="0"/>
-        <v>2479</v>
+        <v>2480</v>
       </c>
       <c r="F37" s="22">
-        <v>20518</v>
+        <v>20519</v>
       </c>
       <c r="G37" s="10">
         <f t="shared" si="1"/>
-        <v>0.92440079293566413</v>
+        <v>0.92444584609839608</v>
       </c>
       <c r="H37" s="6">
         <v>10774</v>
@@ -5913,14 +5913,14 @@
       </c>
       <c r="AD39" s="9">
         <f t="shared" si="10"/>
-        <v>39521</v>
+        <v>39522</v>
       </c>
       <c r="AE39" s="22">
-        <v>224343</v>
+        <v>224344</v>
       </c>
       <c r="AF39" s="10">
         <f t="shared" si="11"/>
-        <v>0.95565144789865131</v>
+        <v>0.9556557076769725</v>
       </c>
       <c r="AG39" s="6">
         <v>132146</v>
@@ -5964,14 +5964,14 @@
       </c>
       <c r="AS39" s="9">
         <f t="shared" si="16"/>
-        <v>50859</v>
+        <v>50861</v>
       </c>
       <c r="AT39" s="22">
-        <v>233363</v>
+        <v>233365</v>
       </c>
       <c r="AU39" s="10">
         <f t="shared" si="17"/>
-        <v>0.94955261412510528</v>
+        <v>0.94956075211282509</v>
       </c>
     </row>
     <row r="40" spans="1:47" x14ac:dyDescent="0.3">
@@ -5989,14 +5989,14 @@
       </c>
       <c r="E40" s="9">
         <f t="shared" si="0"/>
-        <v>75534</v>
+        <v>75580</v>
       </c>
       <c r="F40" s="22">
-        <v>569381</v>
+        <v>569427</v>
       </c>
       <c r="G40" s="10">
         <f t="shared" si="1"/>
-        <v>0.91120496234392656</v>
+        <v>0.91127857812715041</v>
       </c>
       <c r="H40" s="6">
         <v>436886</v>
@@ -6006,14 +6006,14 @@
       </c>
       <c r="J40" s="9">
         <f t="shared" si="2"/>
-        <v>35754</v>
+        <v>35793</v>
       </c>
       <c r="K40" s="22">
-        <v>380931</v>
+        <v>380970</v>
       </c>
       <c r="L40" s="10">
         <f t="shared" si="3"/>
-        <v>0.87192311037661996</v>
+        <v>0.87201237851521907</v>
       </c>
       <c r="M40" s="6">
         <v>700632</v>
@@ -6023,14 +6023,14 @@
       </c>
       <c r="O40" s="9">
         <f t="shared" si="4"/>
-        <v>101804</v>
+        <v>101846</v>
       </c>
       <c r="P40" s="22">
-        <v>624933</v>
+        <v>624975</v>
       </c>
       <c r="Q40" s="10">
         <f t="shared" si="5"/>
-        <v>0.89195611961771659</v>
+        <v>0.892016065495153</v>
       </c>
       <c r="R40" s="6">
         <v>444591</v>
@@ -6040,14 +6040,14 @@
       </c>
       <c r="T40" s="9">
         <f t="shared" si="6"/>
-        <v>39716</v>
+        <v>39748</v>
       </c>
       <c r="U40" s="22">
-        <v>390919</v>
+        <v>390951</v>
       </c>
       <c r="V40" s="10">
         <f t="shared" si="7"/>
-        <v>0.87927780814276491</v>
+        <v>0.87934978440859124</v>
       </c>
       <c r="W40" s="6">
         <v>452148</v>
@@ -6057,14 +6057,14 @@
       </c>
       <c r="Y40" s="9">
         <f t="shared" si="8"/>
-        <v>43440</v>
+        <v>43475</v>
       </c>
       <c r="Z40" s="22">
-        <v>397589</v>
+        <v>397624</v>
       </c>
       <c r="AA40" s="10">
         <f t="shared" si="9"/>
-        <v>0.87933375797305302</v>
+        <v>0.87941116625529692</v>
       </c>
       <c r="AB40" s="6">
         <v>712131</v>
@@ -6074,14 +6074,14 @@
       </c>
       <c r="AD40" s="9">
         <f t="shared" si="10"/>
-        <v>112170</v>
+        <v>112223</v>
       </c>
       <c r="AE40" s="22">
-        <v>635483</v>
+        <v>635536</v>
       </c>
       <c r="AF40" s="10">
         <f t="shared" si="11"/>
-        <v>0.89236811766374446</v>
+        <v>0.89244254217271823</v>
       </c>
       <c r="AG40" s="6">
         <v>463481</v>
@@ -6091,14 +6091,14 @@
       </c>
       <c r="AI40" s="9">
         <f t="shared" si="12"/>
-        <v>52731</v>
+        <v>52772</v>
       </c>
       <c r="AJ40" s="22">
-        <v>402810</v>
+        <v>402851</v>
       </c>
       <c r="AK40" s="10">
         <f t="shared" si="13"/>
-        <v>0.86909711509209653</v>
+        <v>0.86918557610775848</v>
       </c>
       <c r="AL40" s="6">
         <v>472374</v>
@@ -6108,14 +6108,14 @@
       </c>
       <c r="AN40" s="9">
         <f t="shared" si="14"/>
-        <v>57962</v>
+        <v>57994</v>
       </c>
       <c r="AO40" s="22">
-        <v>408018</v>
+        <v>408050</v>
       </c>
       <c r="AP40" s="10">
         <f t="shared" si="15"/>
-        <v>0.86376049486212192</v>
+        <v>0.86382823779462881</v>
       </c>
       <c r="AQ40" s="6">
         <v>750910</v>
@@ -6125,14 +6125,14 @@
       </c>
       <c r="AS40" s="9">
         <f t="shared" si="16"/>
-        <v>138904</v>
+        <v>138963</v>
       </c>
       <c r="AT40" s="22">
-        <v>659062</v>
+        <v>659121</v>
       </c>
       <c r="AU40" s="10">
         <f t="shared" si="17"/>
-        <v>0.87768440958303928</v>
+        <v>0.87776298091648797</v>
       </c>
     </row>
     <row r="41" spans="1:47" x14ac:dyDescent="0.3">
@@ -6506,14 +6506,14 @@
       </c>
       <c r="O43" s="9">
         <f t="shared" si="4"/>
-        <v>34999</v>
+        <v>35000</v>
       </c>
       <c r="P43" s="22">
-        <v>203713</v>
+        <v>203714</v>
       </c>
       <c r="Q43" s="10">
         <f t="shared" si="5"/>
-        <v>0.86725132506013325</v>
+        <v>0.86725558228144495</v>
       </c>
       <c r="R43" s="6">
         <v>144948</v>
@@ -6557,14 +6557,14 @@
       </c>
       <c r="AD43" s="9">
         <f t="shared" si="10"/>
-        <v>41028</v>
+        <v>41030</v>
       </c>
       <c r="AE43" s="22">
-        <v>209295</v>
+        <v>209297</v>
       </c>
       <c r="AF43" s="10">
         <f t="shared" si="11"/>
-        <v>0.86763395170483992</v>
+        <v>0.86764224271945278</v>
       </c>
       <c r="AG43" s="6">
         <v>154073</v>
@@ -6608,14 +6608,14 @@
       </c>
       <c r="AS43" s="9">
         <f t="shared" si="16"/>
-        <v>55145</v>
+        <v>55146</v>
       </c>
       <c r="AT43" s="22">
-        <v>220617</v>
+        <v>220618</v>
       </c>
       <c r="AU43" s="10">
         <f t="shared" si="17"/>
-        <v>0.85120494478783248</v>
+        <v>0.85120880308046087</v>
       </c>
     </row>
     <row r="44" spans="1:47" x14ac:dyDescent="0.3">
@@ -6718,14 +6718,14 @@
       </c>
       <c r="AD44" s="9">
         <f t="shared" si="10"/>
-        <v>36155</v>
+        <v>36156</v>
       </c>
       <c r="AE44" s="22">
-        <v>193269</v>
+        <v>193270</v>
       </c>
       <c r="AF44" s="10">
         <f t="shared" si="11"/>
-        <v>0.8957425705863814</v>
+        <v>0.89574720527984275</v>
       </c>
       <c r="AG44" s="6">
         <v>134716</v>
@@ -6752,14 +6752,14 @@
       </c>
       <c r="AN44" s="9">
         <f t="shared" si="14"/>
-        <v>17426</v>
+        <v>17427</v>
       </c>
       <c r="AO44" s="22">
-        <v>119595</v>
+        <v>119596</v>
       </c>
       <c r="AP44" s="10">
         <f t="shared" si="15"/>
-        <v>0.87395774719934527</v>
+        <v>0.87396505484387221</v>
       </c>
       <c r="AQ44" s="6">
         <v>226630</v>
@@ -6769,14 +6769,14 @@
       </c>
       <c r="AS44" s="9">
         <f t="shared" si="16"/>
-        <v>45591</v>
+        <v>45592</v>
       </c>
       <c r="AT44" s="22">
-        <v>201460</v>
+        <v>201461</v>
       </c>
       <c r="AU44" s="10">
         <f t="shared" si="17"/>
-        <v>0.8889379164276574</v>
+        <v>0.88894232890614655</v>
       </c>
     </row>
     <row r="45" spans="1:47" x14ac:dyDescent="0.3">
@@ -7082,10 +7082,10 @@
       </c>
     </row>
     <row r="47" spans="1:47" s="3" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A47" s="29" t="s">
+      <c r="A47" s="26" t="s">
         <v>42</v>
       </c>
-      <c r="B47" s="29"/>
+      <c r="B47" s="26"/>
       <c r="C47" s="13">
         <f>SUM(C9:C46)</f>
         <v>6783589</v>
@@ -7096,15 +7096,15 @@
       </c>
       <c r="E47" s="11">
         <f>F47-D47</f>
-        <v>989420</v>
+        <v>989511</v>
       </c>
       <c r="F47" s="13">
         <f>SUM(F9:F46)</f>
-        <v>6283423</v>
+        <v>6283514</v>
       </c>
       <c r="G47" s="12">
         <f>F47/C47</f>
-        <v>0.92626823352652998</v>
+        <v>0.92628164825433856</v>
       </c>
       <c r="H47" s="13">
         <f>SUM(H9:H46)</f>
@@ -7116,15 +7116,15 @@
       </c>
       <c r="J47" s="11">
         <f t="shared" si="2"/>
-        <v>240167</v>
+        <v>240224</v>
       </c>
       <c r="K47" s="13">
         <f>SUM(K9:K46)</f>
-        <v>2669693</v>
+        <v>2669750</v>
       </c>
       <c r="L47" s="12">
         <f t="shared" si="3"/>
-        <v>0.84819044605333227</v>
+        <v>0.84820855557207653</v>
       </c>
       <c r="M47" s="13">
         <f>SUM(M9:M46)</f>
@@ -7136,15 +7136,15 @@
       </c>
       <c r="O47" s="11">
         <f t="shared" si="4"/>
-        <v>1297040</v>
+        <v>1297114</v>
       </c>
       <c r="P47" s="13">
         <f>SUM(P9:P46)</f>
-        <v>7192084</v>
+        <v>7192158</v>
       </c>
       <c r="Q47" s="12">
         <f t="shared" si="5"/>
-        <v>0.91770448448820641</v>
+        <v>0.91771392683229647</v>
       </c>
       <c r="R47" s="13">
         <f>SUM(R9:R46)</f>
@@ -7156,15 +7156,15 @@
       </c>
       <c r="T47" s="11">
         <f t="shared" si="6"/>
-        <v>273575</v>
+        <v>273627</v>
       </c>
       <c r="U47" s="13">
         <f>SUM(U9:U46)</f>
-        <v>2762708</v>
+        <v>2762760</v>
       </c>
       <c r="V47" s="12">
         <f t="shared" si="7"/>
-        <v>0.87427994029078027</v>
+        <v>0.8742963960859258</v>
       </c>
       <c r="W47" s="13">
         <f>SUM(W9:W46)</f>
@@ -7176,15 +7176,15 @@
       </c>
       <c r="Y47" s="11">
         <f t="shared" si="8"/>
-        <v>309561</v>
+        <v>309619</v>
       </c>
       <c r="Z47" s="13">
         <f>SUM(Z9:Z46)</f>
-        <v>2821115</v>
+        <v>2821173</v>
       </c>
       <c r="AA47" s="12">
         <f t="shared" si="9"/>
-        <v>0.8784295030676833</v>
+        <v>0.87844756291677772</v>
       </c>
       <c r="AB47" s="13">
         <f>SUM(AB9:AB46)</f>
@@ -7196,15 +7196,15 @@
       </c>
       <c r="AD47" s="11">
         <f t="shared" si="10"/>
-        <v>1416718</v>
+        <v>1416814</v>
       </c>
       <c r="AE47" s="13">
         <f>SUM(AE9:AE46)</f>
-        <v>7335588</v>
+        <v>7335684</v>
       </c>
       <c r="AF47" s="12">
         <f t="shared" si="11"/>
-        <v>0.92029884795598371</v>
+        <v>0.92031089180160375</v>
       </c>
       <c r="AG47" s="13">
         <f>SUM(AG9:AG46)</f>
@@ -7216,15 +7216,15 @@
       </c>
       <c r="AI47" s="11">
         <f t="shared" si="12"/>
-        <v>368763</v>
+        <v>368819</v>
       </c>
       <c r="AJ47" s="13">
         <f>SUM(AJ9:AJ46)</f>
-        <v>2853694</v>
+        <v>2853750</v>
       </c>
       <c r="AK47" s="12">
         <f t="shared" si="13"/>
-        <v>0.86667504886579128</v>
+        <v>0.86669205622633394</v>
       </c>
       <c r="AL47" s="13">
         <f>SUM(AL9:AL46)</f>
@@ -7236,15 +7236,15 @@
       </c>
       <c r="AN47" s="11">
         <f t="shared" si="14"/>
-        <v>405226</v>
+        <v>405277</v>
       </c>
       <c r="AO47" s="13">
         <f>SUM(AO9:AO46)</f>
-        <v>2878401</v>
+        <v>2878452</v>
       </c>
       <c r="AP47" s="12">
         <f t="shared" si="15"/>
-        <v>0.86104651336709637</v>
+        <v>0.86106176953612268</v>
       </c>
       <c r="AQ47" s="13">
         <f>SUM(AQ9:AQ46)</f>
@@ -7256,15 +7256,15 @@
       </c>
       <c r="AS47" s="11">
         <f t="shared" si="16"/>
-        <v>1762842</v>
+        <v>1762950</v>
       </c>
       <c r="AT47" s="13">
         <f>SUM(AT9:AT46)</f>
-        <v>7684545</v>
+        <v>7684653</v>
       </c>
       <c r="AU47" s="12">
         <f t="shared" si="17"/>
-        <v>0.90880777346888164</v>
+        <v>0.90882054601944051</v>
       </c>
     </row>
     <row r="48" spans="1:47" x14ac:dyDescent="0.3">
@@ -7405,17 +7405,22 @@
       <c r="AT57" s="4"/>
     </row>
     <row r="58" spans="1:47" x14ac:dyDescent="0.3">
-      <c r="A58" s="30" t="s">
+      <c r="A58" s="27" t="s">
         <v>43</v>
       </c>
-      <c r="B58" s="30"/>
-      <c r="C58" s="30"/>
-      <c r="D58" s="30"/>
-      <c r="E58" s="30"/>
+      <c r="B58" s="27"/>
+      <c r="C58" s="27"/>
+      <c r="D58" s="27"/>
+      <c r="E58" s="27"/>
       <c r="F58" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="C7:G7"/>
     <mergeCell ref="AQ7:AU7"/>
     <mergeCell ref="A47:B47"/>
     <mergeCell ref="A58:E58"/>
@@ -7426,11 +7431,6 @@
     <mergeCell ref="AG7:AK7"/>
     <mergeCell ref="AL7:AP7"/>
     <mergeCell ref="H7:L7"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A5:C5"/>
-    <mergeCell ref="A7:A8"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="C7:G7"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
chore: sync GST statistics files 2026-08-15
</commit_message>
<xml_diff>
--- a/gstdatabase/GSTR-1-2017-2018.xlsx
+++ b/gstdatabase/GSTR-1-2017-2018.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GSTN\Krishnan Sir\Monthly Report\May-26\GST Statistics Downloads 31st May 26\Downloads\GSTR 1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GSTN\Krishnan Sir\Monthly Report\Jun-26\GST Statistics Downloads 31st May 26\Downloads\GSTR 1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7772CF6D-528E-4F6F-A313-92E513D4D3FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C927B25A-E4B3-4959-B5BD-939701EE9DC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -182,10 +182,10 @@
     <t>Andaman and Nicobar Islands</t>
   </si>
   <si>
-    <t>Data Considered upto 31st May 2026</t>
+    <t>Data Considered upto 30th Jun 2026</t>
   </si>
   <si>
-    <t>Filing %age as on 31st May 2026</t>
+    <t>Filing %age as on 30th Jun 2026</t>
   </si>
 </sst>
 </file>
@@ -997,14 +997,14 @@
       </c>
       <c r="E9" s="9">
         <f t="shared" ref="E9:E44" si="0">F9-D9</f>
-        <v>7346</v>
+        <v>7347</v>
       </c>
       <c r="F9" s="22">
-        <v>46112</v>
+        <v>46113</v>
       </c>
       <c r="G9" s="10">
         <f t="shared" ref="G9:G44" si="1">F9/C9</f>
-        <v>0.87907730435611475</v>
+        <v>0.87909636831569915</v>
       </c>
       <c r="H9" s="6">
         <v>23864</v>
@@ -1014,14 +1014,14 @@
       </c>
       <c r="J9" s="9">
         <f>K9-I9</f>
-        <v>2294</v>
+        <v>2295</v>
       </c>
       <c r="K9" s="22">
-        <v>19632</v>
+        <v>19633</v>
       </c>
       <c r="L9" s="10">
         <f>K9/H9</f>
-        <v>0.82266174991619179</v>
+        <v>0.82270365403955747</v>
       </c>
       <c r="M9" s="6">
         <v>62528</v>
@@ -1031,14 +1031,14 @@
       </c>
       <c r="O9" s="9">
         <f>P9-N9</f>
-        <v>10922</v>
+        <v>10923</v>
       </c>
       <c r="P9" s="22">
-        <v>55852</v>
+        <v>55853</v>
       </c>
       <c r="Q9" s="10">
         <f>P9/M9</f>
-        <v>0.89323183213920165</v>
+        <v>0.89324782497441146</v>
       </c>
       <c r="R9" s="6">
         <v>25413</v>
@@ -1048,14 +1048,14 @@
       </c>
       <c r="T9" s="9">
         <f>U9-S9</f>
-        <v>2805</v>
+        <v>2806</v>
       </c>
       <c r="U9" s="22">
-        <v>21210</v>
+        <v>21211</v>
       </c>
       <c r="V9" s="10">
         <f>U9/R9</f>
-        <v>0.83461220635108013</v>
+        <v>0.8346515562900878</v>
       </c>
       <c r="W9" s="6">
         <v>26079</v>
@@ -1193,14 +1193,14 @@
       </c>
       <c r="O10" s="9">
         <f t="shared" ref="O10:O47" si="4">P10-N10</f>
-        <v>9535</v>
+        <v>9536</v>
       </c>
       <c r="P10" s="22">
-        <v>56454</v>
+        <v>56455</v>
       </c>
       <c r="Q10" s="10">
         <f t="shared" ref="Q10:Q47" si="5">P10/M10</f>
-        <v>0.9151091731370864</v>
+        <v>0.9151253829569953</v>
       </c>
       <c r="R10" s="6">
         <v>21474</v>
@@ -1642,14 +1642,14 @@
       </c>
       <c r="E13" s="9">
         <f t="shared" si="0"/>
-        <v>16193</v>
+        <v>16195</v>
       </c>
       <c r="F13" s="22">
-        <v>75592</v>
+        <v>75594</v>
       </c>
       <c r="G13" s="10">
         <f t="shared" si="1"/>
-        <v>0.88546327749795006</v>
+        <v>0.88548670493147474</v>
       </c>
       <c r="H13" s="6">
         <v>34516</v>
@@ -1676,14 +1676,14 @@
       </c>
       <c r="O13" s="9">
         <f t="shared" si="4"/>
-        <v>21060</v>
+        <v>21062</v>
       </c>
       <c r="P13" s="22">
-        <v>87510</v>
+        <v>87512</v>
       </c>
       <c r="Q13" s="10">
         <f t="shared" si="5"/>
-        <v>0.87441795399588318</v>
+        <v>0.87443793840804174</v>
       </c>
       <c r="R13" s="6">
         <v>34094</v>
@@ -1693,14 +1693,14 @@
       </c>
       <c r="T13" s="9">
         <f t="shared" si="6"/>
-        <v>3416</v>
+        <v>3417</v>
       </c>
       <c r="U13" s="22">
-        <v>26819</v>
+        <v>26820</v>
       </c>
       <c r="V13" s="10">
         <f t="shared" si="7"/>
-        <v>0.78661934651258281</v>
+        <v>0.7866486771866017</v>
       </c>
       <c r="W13" s="6">
         <v>34556</v>
@@ -1710,14 +1710,14 @@
       </c>
       <c r="Y13" s="9">
         <f t="shared" si="8"/>
-        <v>3913</v>
+        <v>3914</v>
       </c>
       <c r="Z13" s="22">
-        <v>27526</v>
+        <v>27527</v>
       </c>
       <c r="AA13" s="10">
         <f t="shared" si="9"/>
-        <v>0.79656210209514988</v>
+        <v>0.79659104062970254</v>
       </c>
       <c r="AB13" s="6">
         <v>99756</v>
@@ -1727,14 +1727,14 @@
       </c>
       <c r="AD13" s="9">
         <f t="shared" si="10"/>
-        <v>22132</v>
+        <v>22133</v>
       </c>
       <c r="AE13" s="22">
-        <v>87329</v>
+        <v>87330</v>
       </c>
       <c r="AF13" s="10">
         <f t="shared" si="11"/>
-        <v>0.87542603953646903</v>
+        <v>0.87543606399615059</v>
       </c>
       <c r="AG13" s="6">
         <v>35615</v>
@@ -1744,14 +1744,14 @@
       </c>
       <c r="AI13" s="9">
         <f t="shared" si="12"/>
-        <v>4638</v>
+        <v>4639</v>
       </c>
       <c r="AJ13" s="22">
-        <v>27778</v>
+        <v>27779</v>
       </c>
       <c r="AK13" s="10">
         <f t="shared" si="13"/>
-        <v>0.77995226730310263</v>
+        <v>0.77998034536010108</v>
       </c>
       <c r="AL13" s="6">
         <v>36218</v>
@@ -1761,14 +1761,14 @@
       </c>
       <c r="AN13" s="9">
         <f t="shared" si="14"/>
-        <v>5093</v>
+        <v>5094</v>
       </c>
       <c r="AO13" s="22">
-        <v>27900</v>
+        <v>27901</v>
       </c>
       <c r="AP13" s="10">
         <f t="shared" si="15"/>
-        <v>0.77033519244574522</v>
+        <v>0.77036280302611959</v>
       </c>
       <c r="AQ13" s="6">
         <v>107596</v>
@@ -1778,14 +1778,14 @@
       </c>
       <c r="AS13" s="9">
         <f t="shared" si="16"/>
-        <v>28029</v>
+        <v>28034</v>
       </c>
       <c r="AT13" s="22">
-        <v>92878</v>
+        <v>92883</v>
       </c>
       <c r="AU13" s="10">
         <f t="shared" si="17"/>
-        <v>0.8632105282724265</v>
+        <v>0.86325699840142756</v>
       </c>
     </row>
     <row r="14" spans="1:48" x14ac:dyDescent="0.3">
@@ -1981,14 +1981,14 @@
       </c>
       <c r="J15" s="9">
         <f t="shared" si="2"/>
-        <v>7988</v>
+        <v>7989</v>
       </c>
       <c r="K15" s="22">
-        <v>139386</v>
+        <v>139387</v>
       </c>
       <c r="L15" s="10">
         <f t="shared" si="3"/>
-        <v>0.88976981117622278</v>
+        <v>0.88977619467105851</v>
       </c>
       <c r="M15" s="6">
         <v>521051</v>
@@ -2015,14 +2015,14 @@
       </c>
       <c r="T15" s="9">
         <f t="shared" si="6"/>
-        <v>9287</v>
+        <v>9288</v>
       </c>
       <c r="U15" s="22">
-        <v>145603</v>
+        <v>145604</v>
       </c>
       <c r="V15" s="10">
         <f t="shared" si="7"/>
-        <v>0.88407662649139318</v>
+        <v>0.88408269832113906</v>
       </c>
       <c r="W15" s="6">
         <v>167887</v>
@@ -2032,14 +2032,14 @@
       </c>
       <c r="Y15" s="9">
         <f t="shared" si="8"/>
-        <v>10221</v>
+        <v>10222</v>
       </c>
       <c r="Z15" s="22">
-        <v>147953</v>
+        <v>147954</v>
       </c>
       <c r="AA15" s="10">
         <f t="shared" si="9"/>
-        <v>0.88126537492480062</v>
+        <v>0.88127133131213253</v>
       </c>
       <c r="AB15" s="6">
         <v>558644</v>
@@ -2066,14 +2066,14 @@
       </c>
       <c r="AI15" s="9">
         <f t="shared" si="12"/>
-        <v>12378</v>
+        <v>12379</v>
       </c>
       <c r="AJ15" s="22">
-        <v>150146</v>
+        <v>150147</v>
       </c>
       <c r="AK15" s="10">
         <f t="shared" si="13"/>
-        <v>0.86595381456617526</v>
+        <v>0.86595958197799161</v>
       </c>
       <c r="AL15" s="6">
         <v>176069</v>
@@ -2083,14 +2083,14 @@
       </c>
       <c r="AN15" s="9">
         <f t="shared" si="14"/>
-        <v>13769</v>
+        <v>13770</v>
       </c>
       <c r="AO15" s="22">
-        <v>151281</v>
+        <v>151282</v>
       </c>
       <c r="AP15" s="10">
         <f t="shared" si="15"/>
-        <v>0.85921428530860056</v>
+        <v>0.85921996490012442</v>
       </c>
       <c r="AQ15" s="6">
         <v>592372</v>
@@ -2125,14 +2125,14 @@
       </c>
       <c r="E16" s="9">
         <f t="shared" si="0"/>
-        <v>69318</v>
+        <v>69322</v>
       </c>
       <c r="F16" s="22">
-        <v>377591</v>
+        <v>377595</v>
       </c>
       <c r="G16" s="10">
         <f t="shared" si="1"/>
-        <v>0.94509980601964838</v>
+        <v>0.94510981790876669</v>
       </c>
       <c r="H16" s="6">
         <v>126607</v>
@@ -2159,14 +2159,14 @@
       </c>
       <c r="O16" s="9">
         <f t="shared" si="4"/>
-        <v>77978</v>
+        <v>77979</v>
       </c>
       <c r="P16" s="22">
-        <v>411132</v>
+        <v>411133</v>
       </c>
       <c r="Q16" s="10">
         <f t="shared" si="5"/>
-        <v>0.94311688371271474</v>
+        <v>0.94311917766425268</v>
       </c>
       <c r="R16" s="6">
         <v>119115</v>
@@ -2210,14 +2210,14 @@
       </c>
       <c r="AD16" s="9">
         <f t="shared" si="10"/>
-        <v>79140</v>
+        <v>79141</v>
       </c>
       <c r="AE16" s="22">
-        <v>412176</v>
+        <v>412177</v>
       </c>
       <c r="AF16" s="10">
         <f t="shared" si="11"/>
-        <v>0.95111685434742477</v>
+        <v>0.95111916189772938</v>
       </c>
       <c r="AG16" s="6">
         <v>121543</v>
@@ -2320,14 +2320,14 @@
       </c>
       <c r="O17" s="9">
         <f t="shared" si="4"/>
-        <v>168606</v>
+        <v>168607</v>
       </c>
       <c r="P17" s="22">
-        <v>800814</v>
+        <v>800815</v>
       </c>
       <c r="Q17" s="10">
         <f t="shared" si="5"/>
-        <v>0.90196383197275232</v>
+        <v>0.90196495828152312</v>
       </c>
       <c r="R17" s="6">
         <v>272330</v>
@@ -2422,14 +2422,14 @@
       </c>
       <c r="AS17" s="9">
         <f t="shared" si="16"/>
-        <v>211266</v>
+        <v>211268</v>
       </c>
       <c r="AT17" s="22">
-        <v>816219</v>
+        <v>816221</v>
       </c>
       <c r="AU17" s="10">
         <f t="shared" si="17"/>
-        <v>0.8938410506823018</v>
+        <v>0.8938432408813799</v>
       </c>
     </row>
     <row r="18" spans="1:47" x14ac:dyDescent="0.3">
@@ -2583,14 +2583,14 @@
       </c>
       <c r="AS18" s="9">
         <f t="shared" si="16"/>
-        <v>69317</v>
+        <v>69318</v>
       </c>
       <c r="AT18" s="22">
-        <v>200042</v>
+        <v>200043</v>
       </c>
       <c r="AU18" s="10">
         <f t="shared" si="17"/>
-        <v>0.83790383721271167</v>
+        <v>0.83790802585228341</v>
       </c>
     </row>
     <row r="19" spans="1:47" x14ac:dyDescent="0.3">
@@ -3388,14 +3388,14 @@
       </c>
       <c r="AS23" s="9">
         <f t="shared" si="16"/>
-        <v>809</v>
+        <v>810</v>
       </c>
       <c r="AT23" s="22">
-        <v>3118</v>
+        <v>3119</v>
       </c>
       <c r="AU23" s="10">
         <f t="shared" si="17"/>
-        <v>0.77025691699604748</v>
+        <v>0.77050395256916993</v>
       </c>
     </row>
     <row r="24" spans="1:47" x14ac:dyDescent="0.3">
@@ -3659,14 +3659,14 @@
       </c>
       <c r="AD25" s="9">
         <f t="shared" si="10"/>
-        <v>3678</v>
+        <v>3679</v>
       </c>
       <c r="AE25" s="22">
-        <v>12355</v>
+        <v>12356</v>
       </c>
       <c r="AF25" s="10">
         <f t="shared" si="11"/>
-        <v>0.80237693206909988</v>
+        <v>0.80244187556825564</v>
       </c>
       <c r="AG25" s="6">
         <v>8752</v>
@@ -3676,14 +3676,14 @@
       </c>
       <c r="AI25" s="9">
         <f t="shared" si="12"/>
-        <v>1958</v>
+        <v>1959</v>
       </c>
       <c r="AJ25" s="22">
-        <v>6316</v>
+        <v>6317</v>
       </c>
       <c r="AK25" s="10">
         <f t="shared" si="13"/>
-        <v>0.72166361974405846</v>
+        <v>0.72177787934186477</v>
       </c>
       <c r="AL25" s="6">
         <v>8845</v>
@@ -3693,14 +3693,14 @@
       </c>
       <c r="AN25" s="9">
         <f t="shared" si="14"/>
-        <v>2103</v>
+        <v>2104</v>
       </c>
       <c r="AO25" s="22">
-        <v>6373</v>
+        <v>6374</v>
       </c>
       <c r="AP25" s="10">
         <f t="shared" si="15"/>
-        <v>0.72052006783493494</v>
+        <v>0.72063312605992091</v>
       </c>
       <c r="AQ25" s="6">
         <v>16327</v>
@@ -3735,14 +3735,14 @@
       </c>
       <c r="E26" s="9">
         <f t="shared" si="0"/>
-        <v>19649</v>
+        <v>19650</v>
       </c>
       <c r="F26" s="22">
-        <v>77928</v>
+        <v>77929</v>
       </c>
       <c r="G26" s="10">
         <f t="shared" si="1"/>
-        <v>0.80104437568742737</v>
+        <v>0.80105465497568951</v>
       </c>
       <c r="H26" s="6">
         <v>56748</v>
@@ -3837,14 +3837,14 @@
       </c>
       <c r="AI26" s="9">
         <f t="shared" si="12"/>
-        <v>10041</v>
+        <v>10042</v>
       </c>
       <c r="AJ26" s="22">
-        <v>39518</v>
+        <v>39519</v>
       </c>
       <c r="AK26" s="10">
         <f t="shared" si="13"/>
-        <v>0.70306717904924565</v>
+        <v>0.70308497011101623</v>
       </c>
       <c r="AL26" s="6">
         <v>57763</v>
@@ -3854,14 +3854,14 @@
       </c>
       <c r="AN26" s="9">
         <f t="shared" si="14"/>
-        <v>10832</v>
+        <v>10833</v>
       </c>
       <c r="AO26" s="22">
-        <v>39844</v>
+        <v>39845</v>
       </c>
       <c r="AP26" s="10">
         <f t="shared" si="15"/>
-        <v>0.68978411786091443</v>
+        <v>0.68980142998112981</v>
       </c>
       <c r="AQ26" s="6">
         <v>122022</v>
@@ -3930,14 +3930,14 @@
       </c>
       <c r="O27" s="9">
         <f t="shared" si="4"/>
-        <v>50598</v>
+        <v>50599</v>
       </c>
       <c r="P27" s="22">
-        <v>384726</v>
+        <v>384727</v>
       </c>
       <c r="Q27" s="10">
         <f t="shared" si="5"/>
-        <v>0.92475320348724011</v>
+        <v>0.92475560715427452</v>
       </c>
       <c r="R27" s="6">
         <v>158774</v>
@@ -3981,14 +3981,14 @@
       </c>
       <c r="AD27" s="9">
         <f t="shared" si="10"/>
-        <v>64102</v>
+        <v>64103</v>
       </c>
       <c r="AE27" s="22">
-        <v>408370</v>
+        <v>408371</v>
       </c>
       <c r="AF27" s="10">
         <f t="shared" si="11"/>
-        <v>0.91997603020554553</v>
+        <v>0.91997828300577622</v>
       </c>
       <c r="AG27" s="6">
         <v>164959</v>
@@ -4032,14 +4032,14 @@
       </c>
       <c r="AS27" s="9">
         <f t="shared" si="16"/>
-        <v>87044</v>
+        <v>87045</v>
       </c>
       <c r="AT27" s="22">
-        <v>430565</v>
+        <v>430566</v>
       </c>
       <c r="AU27" s="10">
         <f t="shared" si="17"/>
-        <v>0.91032005446296049</v>
+        <v>0.91032216870832294</v>
       </c>
     </row>
     <row r="28" spans="1:47" x14ac:dyDescent="0.3">
@@ -4057,14 +4057,14 @@
       </c>
       <c r="E28" s="9">
         <f t="shared" si="0"/>
-        <v>11663</v>
+        <v>11664</v>
       </c>
       <c r="F28" s="22">
-        <v>76029</v>
+        <v>76030</v>
       </c>
       <c r="G28" s="10">
         <f t="shared" si="1"/>
-        <v>0.91733832046332042</v>
+        <v>0.91735038610038611</v>
       </c>
       <c r="H28" s="6">
         <v>43355</v>
@@ -4091,14 +4091,14 @@
       </c>
       <c r="O28" s="9">
         <f t="shared" si="4"/>
-        <v>17295</v>
+        <v>17296</v>
       </c>
       <c r="P28" s="22">
-        <v>90750</v>
+        <v>90751</v>
       </c>
       <c r="Q28" s="10">
         <f t="shared" si="5"/>
-        <v>0.90132591746536228</v>
+        <v>0.901335849431395</v>
       </c>
       <c r="R28" s="6">
         <v>44777</v>
@@ -4142,14 +4142,14 @@
       </c>
       <c r="AD28" s="9">
         <f t="shared" si="10"/>
-        <v>20856</v>
+        <v>20857</v>
       </c>
       <c r="AE28" s="22">
-        <v>97492</v>
+        <v>97493</v>
       </c>
       <c r="AF28" s="10">
         <f t="shared" si="11"/>
-        <v>0.90197711103092881</v>
+        <v>0.90198636283734401</v>
       </c>
       <c r="AG28" s="6">
         <v>47997</v>
@@ -4193,14 +4193,14 @@
       </c>
       <c r="AS28" s="9">
         <f t="shared" si="16"/>
-        <v>29725</v>
+        <v>29726</v>
       </c>
       <c r="AT28" s="22">
-        <v>103465</v>
+        <v>103466</v>
       </c>
       <c r="AU28" s="10">
         <f t="shared" si="17"/>
-        <v>0.88267913357277528</v>
+        <v>0.88268766475852478</v>
       </c>
     </row>
     <row r="29" spans="1:47" x14ac:dyDescent="0.3">
@@ -4515,14 +4515,14 @@
       </c>
       <c r="AS30" s="9">
         <f t="shared" si="16"/>
-        <v>27514</v>
+        <v>27515</v>
       </c>
       <c r="AT30" s="22">
-        <v>81680</v>
+        <v>81681</v>
       </c>
       <c r="AU30" s="10">
         <f t="shared" si="17"/>
-        <v>0.86572194723844453</v>
+        <v>0.86573254618490925</v>
       </c>
     </row>
     <row r="31" spans="1:47" x14ac:dyDescent="0.3">
@@ -4540,14 +4540,14 @@
       </c>
       <c r="E31" s="9">
         <f t="shared" si="0"/>
-        <v>43650</v>
+        <v>43652</v>
       </c>
       <c r="F31" s="22">
-        <v>240842</v>
+        <v>240844</v>
       </c>
       <c r="G31" s="10">
         <f t="shared" si="1"/>
-        <v>0.93600665350474921</v>
+        <v>0.93601442629067111</v>
       </c>
       <c r="H31" s="6">
         <v>94897</v>
@@ -4557,14 +4557,14 @@
       </c>
       <c r="J31" s="9">
         <f t="shared" si="2"/>
-        <v>7083</v>
+        <v>7085</v>
       </c>
       <c r="K31" s="22">
-        <v>80252</v>
+        <v>80254</v>
       </c>
       <c r="L31" s="10">
         <f t="shared" si="3"/>
-        <v>0.84567478423975473</v>
+        <v>0.84569585972159289</v>
       </c>
       <c r="M31" s="6">
         <v>290350</v>
@@ -4574,14 +4574,14 @@
       </c>
       <c r="O31" s="9">
         <f t="shared" si="4"/>
-        <v>53550</v>
+        <v>53551</v>
       </c>
       <c r="P31" s="22">
-        <v>265707</v>
+        <v>265708</v>
       </c>
       <c r="Q31" s="10">
         <f t="shared" si="5"/>
-        <v>0.9151265713793697</v>
+        <v>0.91513001549853623</v>
       </c>
       <c r="R31" s="6">
         <v>95518</v>
@@ -4591,14 +4591,14 @@
       </c>
       <c r="T31" s="9">
         <f t="shared" si="6"/>
-        <v>8297</v>
+        <v>8298</v>
       </c>
       <c r="U31" s="22">
-        <v>82234</v>
+        <v>82235</v>
       </c>
       <c r="V31" s="10">
         <f t="shared" si="7"/>
-        <v>0.86092673632194983</v>
+        <v>0.86093720555288011</v>
       </c>
       <c r="W31" s="6">
         <v>97097</v>
@@ -4608,14 +4608,14 @@
       </c>
       <c r="Y31" s="9">
         <f t="shared" si="8"/>
-        <v>9333</v>
+        <v>9334</v>
       </c>
       <c r="Z31" s="22">
-        <v>83635</v>
+        <v>83636</v>
       </c>
       <c r="AA31" s="10">
         <f t="shared" si="9"/>
-        <v>0.86135513970565514</v>
+        <v>0.86136543868502635</v>
       </c>
       <c r="AB31" s="6">
         <v>286853</v>
@@ -4625,14 +4625,14 @@
       </c>
       <c r="AD31" s="9">
         <f t="shared" si="10"/>
-        <v>56142</v>
+        <v>56143</v>
       </c>
       <c r="AE31" s="22">
-        <v>261925</v>
+        <v>261926</v>
       </c>
       <c r="AF31" s="10">
         <f t="shared" si="11"/>
-        <v>0.91309834653986532</v>
+        <v>0.91310183264598943</v>
       </c>
       <c r="AG31" s="6">
         <v>99962</v>
@@ -4642,14 +4642,14 @@
       </c>
       <c r="AI31" s="9">
         <f t="shared" si="12"/>
-        <v>11512</v>
+        <v>11513</v>
       </c>
       <c r="AJ31" s="22">
-        <v>84145</v>
+        <v>84146</v>
       </c>
       <c r="AK31" s="10">
         <f t="shared" si="13"/>
-        <v>0.84176987255156954</v>
+        <v>0.8417798763530141</v>
       </c>
       <c r="AL31" s="6">
         <v>100963</v>
@@ -4659,14 +4659,14 @@
       </c>
       <c r="AN31" s="9">
         <f t="shared" si="14"/>
-        <v>12800</v>
+        <v>12801</v>
       </c>
       <c r="AO31" s="22">
-        <v>84479</v>
+        <v>84480</v>
       </c>
       <c r="AP31" s="10">
         <f t="shared" si="15"/>
-        <v>0.83673226825668812</v>
+        <v>0.83674217287521169</v>
       </c>
       <c r="AQ31" s="6">
         <v>304929</v>
@@ -4701,14 +4701,14 @@
       </c>
       <c r="E32" s="9">
         <f t="shared" si="0"/>
-        <v>68658</v>
+        <v>68664</v>
       </c>
       <c r="F32" s="22">
-        <v>540580</v>
+        <v>540586</v>
       </c>
       <c r="G32" s="10">
         <f t="shared" si="1"/>
-        <v>0.95756006228090529</v>
+        <v>0.95757069042174237</v>
       </c>
       <c r="H32" s="6">
         <v>224696</v>
@@ -4718,14 +4718,14 @@
       </c>
       <c r="J32" s="9">
         <f t="shared" si="2"/>
-        <v>8455</v>
+        <v>8458</v>
       </c>
       <c r="K32" s="22">
-        <v>204575</v>
+        <v>204578</v>
       </c>
       <c r="L32" s="10">
         <f t="shared" si="3"/>
-        <v>0.91045234450101475</v>
+        <v>0.91046569587353576</v>
       </c>
       <c r="M32" s="6">
         <v>682019</v>
@@ -4735,14 +4735,14 @@
       </c>
       <c r="O32" s="9">
         <f t="shared" si="4"/>
-        <v>94826</v>
+        <v>94830</v>
       </c>
       <c r="P32" s="22">
-        <v>656095</v>
+        <v>656099</v>
       </c>
       <c r="Q32" s="10">
         <f t="shared" si="5"/>
-        <v>0.96198932874304088</v>
+        <v>0.96199519368228747</v>
       </c>
       <c r="R32" s="6">
         <v>225967</v>
@@ -4786,14 +4786,14 @@
       </c>
       <c r="AD32" s="9">
         <f t="shared" si="10"/>
-        <v>100363</v>
+        <v>100364</v>
       </c>
       <c r="AE32" s="22">
-        <v>678197</v>
+        <v>678198</v>
       </c>
       <c r="AF32" s="10">
         <f t="shared" si="11"/>
-        <v>0.97042077986003095</v>
+        <v>0.97042221074335822</v>
       </c>
       <c r="AG32" s="6">
         <v>232401</v>
@@ -4803,14 +4803,14 @@
       </c>
       <c r="AI32" s="9">
         <f t="shared" si="12"/>
-        <v>13767</v>
+        <v>13770</v>
       </c>
       <c r="AJ32" s="22">
-        <v>218606</v>
+        <v>218609</v>
       </c>
       <c r="AK32" s="10">
         <f t="shared" si="13"/>
-        <v>0.94064139138816094</v>
+        <v>0.94065430011058471</v>
       </c>
       <c r="AL32" s="6">
         <v>234200</v>
@@ -4820,14 +4820,14 @@
       </c>
       <c r="AN32" s="9">
         <f t="shared" si="14"/>
-        <v>14852</v>
+        <v>14853</v>
       </c>
       <c r="AO32" s="22">
-        <v>219620</v>
+        <v>219621</v>
       </c>
       <c r="AP32" s="10">
         <f t="shared" si="15"/>
-        <v>0.93774551665243377</v>
+        <v>0.93774978650725871</v>
       </c>
       <c r="AQ32" s="6">
         <v>733311</v>
@@ -4837,14 +4837,14 @@
       </c>
       <c r="AS32" s="9">
         <f t="shared" si="16"/>
-        <v>118431</v>
+        <v>118433</v>
       </c>
       <c r="AT32" s="22">
-        <v>708215</v>
+        <v>708217</v>
       </c>
       <c r="AU32" s="10">
         <f t="shared" si="17"/>
-        <v>0.96577713957652345</v>
+        <v>0.9657798669323111</v>
       </c>
     </row>
     <row r="33" spans="1:47" x14ac:dyDescent="0.3">
@@ -5184,14 +5184,14 @@
       </c>
       <c r="E35" s="9">
         <f t="shared" si="0"/>
-        <v>145164</v>
+        <v>145166</v>
       </c>
       <c r="F35" s="22">
-        <v>864300</v>
+        <v>864302</v>
       </c>
       <c r="G35" s="10">
         <f t="shared" si="1"/>
-        <v>0.94470166970527669</v>
+        <v>0.94470385575565208</v>
       </c>
       <c r="H35" s="6">
         <v>336894</v>
@@ -5201,14 +5201,14 @@
       </c>
       <c r="J35" s="9">
         <f t="shared" si="2"/>
-        <v>22986</v>
+        <v>22988</v>
       </c>
       <c r="K35" s="22">
-        <v>297055</v>
+        <v>297057</v>
       </c>
       <c r="L35" s="10">
         <f t="shared" si="3"/>
-        <v>0.88174618722803022</v>
+        <v>0.88175212381342505</v>
       </c>
       <c r="M35" s="6">
         <v>1060520</v>
@@ -5218,14 +5218,14 @@
       </c>
       <c r="O35" s="9">
         <f t="shared" si="4"/>
-        <v>190490</v>
+        <v>190492</v>
       </c>
       <c r="P35" s="22">
-        <v>1004073</v>
+        <v>1004075</v>
       </c>
       <c r="Q35" s="10">
         <f t="shared" si="5"/>
-        <v>0.94677422396560174</v>
+        <v>0.94677610983291216</v>
       </c>
       <c r="R35" s="6">
         <v>338572</v>
@@ -5235,14 +5235,14 @@
       </c>
       <c r="T35" s="9">
         <f t="shared" si="6"/>
-        <v>26622</v>
+        <v>26624</v>
       </c>
       <c r="U35" s="22">
-        <v>308482</v>
+        <v>308484</v>
       </c>
       <c r="V35" s="10">
         <f t="shared" si="7"/>
-        <v>0.91112673227555729</v>
+        <v>0.91113263943858325</v>
       </c>
       <c r="W35" s="6">
         <v>341709</v>
@@ -5252,14 +5252,14 @@
       </c>
       <c r="Y35" s="9">
         <f t="shared" si="8"/>
-        <v>30173</v>
+        <v>30175</v>
       </c>
       <c r="Z35" s="22">
-        <v>313380</v>
+        <v>313382</v>
       </c>
       <c r="AA35" s="10">
         <f t="shared" si="9"/>
-        <v>0.91709612565077303</v>
+        <v>0.91710197858411691</v>
       </c>
       <c r="AB35" s="6">
         <v>1094504</v>
@@ -5286,14 +5286,14 @@
       </c>
       <c r="AI35" s="9">
         <f t="shared" si="12"/>
-        <v>36074</v>
+        <v>36075</v>
       </c>
       <c r="AJ35" s="22">
-        <v>316478</v>
+        <v>316479</v>
       </c>
       <c r="AK35" s="10">
         <f t="shared" si="13"/>
-        <v>0.908172108425783</v>
+        <v>0.90817497804739467</v>
       </c>
       <c r="AL35" s="6">
         <v>352081</v>
@@ -5303,14 +5303,14 @@
       </c>
       <c r="AN35" s="9">
         <f t="shared" si="14"/>
-        <v>39183</v>
+        <v>39185</v>
       </c>
       <c r="AO35" s="22">
-        <v>318223</v>
+        <v>318225</v>
       </c>
       <c r="AP35" s="10">
         <f t="shared" si="15"/>
-        <v>0.90383462896322153</v>
+        <v>0.90384030947424032</v>
       </c>
       <c r="AQ35" s="6">
         <v>1148243</v>
@@ -5320,14 +5320,14 @@
       </c>
       <c r="AS35" s="9">
         <f t="shared" si="16"/>
-        <v>254038</v>
+        <v>254041</v>
       </c>
       <c r="AT35" s="22">
-        <v>1087097</v>
+        <v>1087100</v>
       </c>
       <c r="AU35" s="10">
         <f t="shared" si="17"/>
-        <v>0.94674820573693896</v>
+        <v>0.94675081842432307</v>
       </c>
     </row>
     <row r="36" spans="1:47" x14ac:dyDescent="0.3">
@@ -5345,14 +5345,14 @@
       </c>
       <c r="E36" s="9">
         <f t="shared" si="0"/>
-        <v>76405</v>
+        <v>76412</v>
       </c>
       <c r="F36" s="22">
-        <v>460724</v>
+        <v>460731</v>
       </c>
       <c r="G36" s="10">
         <f t="shared" si="1"/>
-        <v>0.91521174715488662</v>
+        <v>0.91522565240451559</v>
       </c>
       <c r="H36" s="6">
         <v>312358</v>
@@ -5362,14 +5362,14 @@
       </c>
       <c r="J36" s="9">
         <f t="shared" si="2"/>
-        <v>32461</v>
+        <v>32464</v>
       </c>
       <c r="K36" s="22">
-        <v>276704</v>
+        <v>276707</v>
       </c>
       <c r="L36" s="10">
         <f t="shared" si="3"/>
-        <v>0.88585533266316219</v>
+        <v>0.88586493702738522</v>
       </c>
       <c r="M36" s="6">
         <v>553919</v>
@@ -5379,14 +5379,14 @@
       </c>
       <c r="O36" s="9">
         <f t="shared" si="4"/>
-        <v>94053</v>
+        <v>94059</v>
       </c>
       <c r="P36" s="22">
-        <v>494793</v>
+        <v>494799</v>
       </c>
       <c r="Q36" s="10">
         <f t="shared" si="5"/>
-        <v>0.89325876166009832</v>
+        <v>0.89326959356873481</v>
       </c>
       <c r="R36" s="6">
         <v>318679</v>
@@ -5396,14 +5396,14 @@
       </c>
       <c r="T36" s="9">
         <f t="shared" si="6"/>
-        <v>35610</v>
+        <v>35614</v>
       </c>
       <c r="U36" s="22">
-        <v>284065</v>
+        <v>284069</v>
       </c>
       <c r="V36" s="10">
         <f t="shared" si="7"/>
-        <v>0.89138286488912044</v>
+        <v>0.89139541670458355</v>
       </c>
       <c r="W36" s="6">
         <v>324721</v>
@@ -5413,14 +5413,14 @@
       </c>
       <c r="Y36" s="9">
         <f t="shared" si="8"/>
-        <v>38954</v>
+        <v>38959</v>
       </c>
       <c r="Z36" s="22">
-        <v>289570</v>
+        <v>289575</v>
       </c>
       <c r="AA36" s="10">
         <f t="shared" si="9"/>
-        <v>0.89175014858909651</v>
+        <v>0.89176554642292927</v>
       </c>
       <c r="AB36" s="6">
         <v>556414</v>
@@ -5430,14 +5430,14 @@
       </c>
       <c r="AD36" s="9">
         <f t="shared" si="10"/>
-        <v>102224</v>
+        <v>102232</v>
       </c>
       <c r="AE36" s="22">
-        <v>499751</v>
+        <v>499759</v>
       </c>
       <c r="AF36" s="10">
         <f t="shared" si="11"/>
-        <v>0.89816395705356089</v>
+        <v>0.89817833483700982</v>
       </c>
       <c r="AG36" s="6">
         <v>333690</v>
@@ -5447,14 +5447,14 @@
       </c>
       <c r="AI36" s="9">
         <f t="shared" si="12"/>
-        <v>47419</v>
+        <v>47427</v>
       </c>
       <c r="AJ36" s="22">
-        <v>293778</v>
+        <v>293786</v>
       </c>
       <c r="AK36" s="10">
         <f t="shared" si="13"/>
-        <v>0.88039198058077861</v>
+        <v>0.88041595492822677</v>
       </c>
       <c r="AL36" s="6">
         <v>339216</v>
@@ -5464,14 +5464,14 @@
       </c>
       <c r="AN36" s="9">
         <f t="shared" si="14"/>
-        <v>52331</v>
+        <v>52337</v>
       </c>
       <c r="AO36" s="22">
-        <v>296767</v>
+        <v>296773</v>
       </c>
       <c r="AP36" s="10">
         <f t="shared" si="15"/>
-        <v>0.87486144521484832</v>
+        <v>0.87487913305976128</v>
       </c>
       <c r="AQ36" s="6">
         <v>590015</v>
@@ -5481,14 +5481,14 @@
       </c>
       <c r="AS36" s="9">
         <f t="shared" si="16"/>
-        <v>131196</v>
+        <v>131203</v>
       </c>
       <c r="AT36" s="22">
-        <v>521178</v>
+        <v>521185</v>
       </c>
       <c r="AU36" s="10">
         <f t="shared" si="17"/>
-        <v>0.88333008482835185</v>
+        <v>0.88334194893350171</v>
       </c>
     </row>
     <row r="37" spans="1:47" x14ac:dyDescent="0.3">
@@ -5828,14 +5828,14 @@
       </c>
       <c r="E39" s="9">
         <f t="shared" si="0"/>
-        <v>27788</v>
+        <v>27790</v>
       </c>
       <c r="F39" s="22">
-        <v>207439</v>
+        <v>207441</v>
       </c>
       <c r="G39" s="10">
         <f t="shared" si="1"/>
-        <v>0.96067707127309776</v>
+        <v>0.96068633353401567</v>
       </c>
       <c r="H39" s="6">
         <v>127093</v>
@@ -5845,14 +5845,14 @@
       </c>
       <c r="J39" s="9">
         <f t="shared" si="2"/>
-        <v>11713</v>
+        <v>11715</v>
       </c>
       <c r="K39" s="22">
-        <v>119556</v>
+        <v>119558</v>
       </c>
       <c r="L39" s="10">
         <f t="shared" si="3"/>
-        <v>0.94069696993540164</v>
+        <v>0.94071270644331317</v>
       </c>
       <c r="M39" s="6">
         <v>233233</v>
@@ -5862,14 +5862,14 @@
       </c>
       <c r="O39" s="9">
         <f t="shared" si="4"/>
-        <v>35024</v>
+        <v>35025</v>
       </c>
       <c r="P39" s="22">
-        <v>222456</v>
+        <v>222457</v>
       </c>
       <c r="Q39" s="10">
         <f t="shared" si="5"/>
-        <v>0.95379298812775204</v>
+        <v>0.95379727568568773</v>
       </c>
       <c r="R39" s="6">
         <v>127401</v>
@@ -5879,14 +5879,14 @@
       </c>
       <c r="T39" s="9">
         <f t="shared" si="6"/>
-        <v>13244</v>
+        <v>13246</v>
       </c>
       <c r="U39" s="22">
-        <v>121412</v>
+        <v>121414</v>
       </c>
       <c r="V39" s="10">
         <f t="shared" si="7"/>
-        <v>0.95299094983555854</v>
+        <v>0.95300664829946391</v>
       </c>
       <c r="W39" s="6">
         <v>129531</v>
@@ -5896,14 +5896,14 @@
       </c>
       <c r="Y39" s="9">
         <f t="shared" si="8"/>
-        <v>14730</v>
+        <v>14731</v>
       </c>
       <c r="Z39" s="22">
-        <v>123692</v>
+        <v>123693</v>
       </c>
       <c r="AA39" s="10">
         <f t="shared" si="9"/>
-        <v>0.95492198778670745</v>
+        <v>0.95492970794636034</v>
       </c>
       <c r="AB39" s="6">
         <v>234754</v>
@@ -5913,14 +5913,14 @@
       </c>
       <c r="AD39" s="9">
         <f t="shared" si="10"/>
-        <v>39522</v>
+        <v>39524</v>
       </c>
       <c r="AE39" s="22">
-        <v>224344</v>
+        <v>224346</v>
       </c>
       <c r="AF39" s="10">
         <f t="shared" si="11"/>
-        <v>0.9556557076769725</v>
+        <v>0.95566422723361477</v>
       </c>
       <c r="AG39" s="6">
         <v>132146</v>
@@ -5930,14 +5930,14 @@
       </c>
       <c r="AI39" s="9">
         <f t="shared" si="12"/>
-        <v>17567</v>
+        <v>17568</v>
       </c>
       <c r="AJ39" s="22">
-        <v>125425</v>
+        <v>125426</v>
       </c>
       <c r="AK39" s="10">
         <f t="shared" si="13"/>
-        <v>0.94913958803141985</v>
+        <v>0.94914715541900629</v>
       </c>
       <c r="AL39" s="6">
         <v>133611</v>
@@ -5947,14 +5947,14 @@
       </c>
       <c r="AN39" s="9">
         <f t="shared" si="14"/>
-        <v>19246</v>
+        <v>19247</v>
       </c>
       <c r="AO39" s="22">
-        <v>126543</v>
+        <v>126544</v>
       </c>
       <c r="AP39" s="10">
         <f t="shared" si="15"/>
-        <v>0.94710016390866025</v>
+        <v>0.94710764832236871</v>
       </c>
       <c r="AQ39" s="6">
         <v>245761</v>
@@ -5964,14 +5964,14 @@
       </c>
       <c r="AS39" s="9">
         <f t="shared" si="16"/>
-        <v>50861</v>
+        <v>50862</v>
       </c>
       <c r="AT39" s="22">
-        <v>233365</v>
+        <v>233366</v>
       </c>
       <c r="AU39" s="10">
         <f t="shared" si="17"/>
-        <v>0.94956075211282509</v>
+        <v>0.94956482110668494</v>
       </c>
     </row>
     <row r="40" spans="1:47" x14ac:dyDescent="0.3">
@@ -5989,14 +5989,14 @@
       </c>
       <c r="E40" s="9">
         <f t="shared" si="0"/>
-        <v>75580</v>
+        <v>75604</v>
       </c>
       <c r="F40" s="22">
-        <v>569427</v>
+        <v>569451</v>
       </c>
       <c r="G40" s="10">
         <f t="shared" si="1"/>
-        <v>0.91127857812715041</v>
+        <v>0.91131698636187597</v>
       </c>
       <c r="H40" s="6">
         <v>436886</v>
@@ -6006,14 +6006,14 @@
       </c>
       <c r="J40" s="9">
         <f t="shared" si="2"/>
-        <v>35793</v>
+        <v>35818</v>
       </c>
       <c r="K40" s="22">
-        <v>380970</v>
+        <v>380995</v>
       </c>
       <c r="L40" s="10">
         <f t="shared" si="3"/>
-        <v>0.87201237851521907</v>
+        <v>0.87206960168098768</v>
       </c>
       <c r="M40" s="6">
         <v>700632</v>
@@ -6023,14 +6023,14 @@
       </c>
       <c r="O40" s="9">
         <f t="shared" si="4"/>
-        <v>101846</v>
+        <v>101870</v>
       </c>
       <c r="P40" s="22">
-        <v>624975</v>
+        <v>624999</v>
       </c>
       <c r="Q40" s="10">
         <f t="shared" si="5"/>
-        <v>0.892016065495153</v>
+        <v>0.89205032028225939</v>
       </c>
       <c r="R40" s="6">
         <v>444591</v>
@@ -6040,14 +6040,14 @@
       </c>
       <c r="T40" s="9">
         <f t="shared" si="6"/>
-        <v>39748</v>
+        <v>39760</v>
       </c>
       <c r="U40" s="22">
-        <v>390951</v>
+        <v>390963</v>
       </c>
       <c r="V40" s="10">
         <f t="shared" si="7"/>
-        <v>0.87934978440859124</v>
+        <v>0.8793767755082762</v>
       </c>
       <c r="W40" s="6">
         <v>452148</v>
@@ -6057,14 +6057,14 @@
       </c>
       <c r="Y40" s="9">
         <f t="shared" si="8"/>
-        <v>43475</v>
+        <v>43487</v>
       </c>
       <c r="Z40" s="22">
-        <v>397624</v>
+        <v>397636</v>
       </c>
       <c r="AA40" s="10">
         <f t="shared" si="9"/>
-        <v>0.87941116625529692</v>
+        <v>0.8794377062377805</v>
       </c>
       <c r="AB40" s="6">
         <v>712131</v>
@@ -6074,14 +6074,14 @@
       </c>
       <c r="AD40" s="9">
         <f t="shared" si="10"/>
-        <v>112223</v>
+        <v>112242</v>
       </c>
       <c r="AE40" s="22">
-        <v>635536</v>
+        <v>635555</v>
       </c>
       <c r="AF40" s="10">
         <f t="shared" si="11"/>
-        <v>0.89244254217271823</v>
+        <v>0.8924692226570673</v>
       </c>
       <c r="AG40" s="6">
         <v>463481</v>
@@ -6091,14 +6091,14 @@
       </c>
       <c r="AI40" s="9">
         <f t="shared" si="12"/>
-        <v>52772</v>
+        <v>52783</v>
       </c>
       <c r="AJ40" s="22">
-        <v>402851</v>
+        <v>402862</v>
       </c>
       <c r="AK40" s="10">
         <f t="shared" si="13"/>
-        <v>0.86918557610775848</v>
+        <v>0.86920930955098485</v>
       </c>
       <c r="AL40" s="6">
         <v>472374</v>
@@ -6108,14 +6108,14 @@
       </c>
       <c r="AN40" s="9">
         <f t="shared" si="14"/>
-        <v>57994</v>
+        <v>58007</v>
       </c>
       <c r="AO40" s="22">
-        <v>408050</v>
+        <v>408063</v>
       </c>
       <c r="AP40" s="10">
         <f t="shared" si="15"/>
-        <v>0.86382823779462881</v>
+        <v>0.86385575836095974</v>
       </c>
       <c r="AQ40" s="6">
         <v>750910</v>
@@ -6125,14 +6125,14 @@
       </c>
       <c r="AS40" s="9">
         <f t="shared" si="16"/>
-        <v>138963</v>
+        <v>138990</v>
       </c>
       <c r="AT40" s="22">
-        <v>659121</v>
+        <v>659148</v>
       </c>
       <c r="AU40" s="10">
         <f t="shared" si="17"/>
-        <v>0.87776298091648797</v>
+        <v>0.87779893728942215</v>
       </c>
     </row>
     <row r="41" spans="1:47" x14ac:dyDescent="0.3">
@@ -6184,14 +6184,14 @@
       </c>
       <c r="O41" s="9">
         <f t="shared" si="4"/>
-        <v>2593</v>
+        <v>2594</v>
       </c>
       <c r="P41" s="22">
-        <v>14242</v>
+        <v>14243</v>
       </c>
       <c r="Q41" s="10">
         <f t="shared" si="5"/>
-        <v>0.91482528263103802</v>
+        <v>0.91488951695786225</v>
       </c>
       <c r="R41" s="6">
         <v>9544</v>
@@ -6235,14 +6235,14 @@
       </c>
       <c r="AD41" s="9">
         <f t="shared" si="10"/>
-        <v>2914</v>
+        <v>2915</v>
       </c>
       <c r="AE41" s="22">
-        <v>14700</v>
+        <v>14701</v>
       </c>
       <c r="AF41" s="10">
         <f t="shared" si="11"/>
-        <v>0.92018779342723001</v>
+        <v>0.9202503912363067</v>
       </c>
       <c r="AG41" s="6">
         <v>9858</v>
@@ -6286,14 +6286,14 @@
       </c>
       <c r="AS41" s="9">
         <f t="shared" si="16"/>
-        <v>3624</v>
+        <v>3625</v>
       </c>
       <c r="AT41" s="22">
-        <v>15378</v>
+        <v>15379</v>
       </c>
       <c r="AU41" s="10">
         <f t="shared" si="17"/>
-        <v>0.91064132172677204</v>
+        <v>0.91070053887605851</v>
       </c>
     </row>
     <row r="42" spans="1:47" x14ac:dyDescent="0.3">
@@ -6684,14 +6684,14 @@
       </c>
       <c r="T44" s="9">
         <f t="shared" si="6"/>
-        <v>11752</v>
+        <v>11753</v>
       </c>
       <c r="U44" s="22">
-        <v>113812</v>
+        <v>113813</v>
       </c>
       <c r="V44" s="10">
         <f t="shared" si="7"/>
-        <v>0.88095238095238093</v>
+        <v>0.88096012136974422</v>
       </c>
       <c r="W44" s="6">
         <v>132744</v>
@@ -7096,15 +7096,15 @@
       </c>
       <c r="E47" s="11">
         <f>F47-D47</f>
-        <v>989511</v>
+        <v>989563</v>
       </c>
       <c r="F47" s="13">
         <f>SUM(F9:F46)</f>
-        <v>6283514</v>
+        <v>6283566</v>
       </c>
       <c r="G47" s="12">
         <f>F47/C47</f>
-        <v>0.92628164825433856</v>
+        <v>0.92628931381308621</v>
       </c>
       <c r="H47" s="13">
         <f>SUM(H9:H46)</f>
@@ -7116,15 +7116,15 @@
       </c>
       <c r="J47" s="11">
         <f t="shared" si="2"/>
-        <v>240224</v>
+        <v>240263</v>
       </c>
       <c r="K47" s="13">
         <f>SUM(K9:K46)</f>
-        <v>2669750</v>
+        <v>2669789</v>
       </c>
       <c r="L47" s="12">
         <f t="shared" si="3"/>
-        <v>0.84820855557207653</v>
+        <v>0.84822094629542788</v>
       </c>
       <c r="M47" s="13">
         <f>SUM(M9:M46)</f>
@@ -7136,15 +7136,15 @@
       </c>
       <c r="O47" s="11">
         <f t="shared" si="4"/>
-        <v>1297114</v>
+        <v>1297161</v>
       </c>
       <c r="P47" s="13">
         <f>SUM(P9:P46)</f>
-        <v>7192158</v>
+        <v>7192205</v>
       </c>
       <c r="Q47" s="12">
         <f t="shared" si="5"/>
-        <v>0.91771392683229647</v>
+        <v>0.91771992399678604</v>
       </c>
       <c r="R47" s="13">
         <f>SUM(R9:R46)</f>
@@ -7156,15 +7156,15 @@
       </c>
       <c r="T47" s="11">
         <f t="shared" si="6"/>
-        <v>273627</v>
+        <v>273652</v>
       </c>
       <c r="U47" s="13">
         <f>SUM(U9:U46)</f>
-        <v>2762760</v>
+        <v>2762785</v>
       </c>
       <c r="V47" s="12">
         <f t="shared" si="7"/>
-        <v>0.8742963960859258</v>
+        <v>0.87430430752589972</v>
       </c>
       <c r="W47" s="13">
         <f>SUM(W9:W46)</f>
@@ -7176,15 +7176,15 @@
       </c>
       <c r="Y47" s="11">
         <f t="shared" si="8"/>
-        <v>309619</v>
+        <v>309642</v>
       </c>
       <c r="Z47" s="13">
         <f>SUM(Z9:Z46)</f>
-        <v>2821173</v>
+        <v>2821196</v>
       </c>
       <c r="AA47" s="12">
         <f t="shared" si="9"/>
-        <v>0.87844756291677772</v>
+        <v>0.87845472458107376</v>
       </c>
       <c r="AB47" s="13">
         <f>SUM(AB9:AB46)</f>
@@ -7196,15 +7196,15 @@
       </c>
       <c r="AD47" s="11">
         <f t="shared" si="10"/>
-        <v>1416814</v>
+        <v>1416851</v>
       </c>
       <c r="AE47" s="13">
         <f>SUM(AE9:AE46)</f>
-        <v>7335684</v>
+        <v>7335721</v>
       </c>
       <c r="AF47" s="12">
         <f t="shared" si="11"/>
-        <v>0.92031089180160375</v>
+        <v>0.92031553370043639</v>
       </c>
       <c r="AG47" s="13">
         <f>SUM(AG9:AG46)</f>
@@ -7216,15 +7216,15 @@
       </c>
       <c r="AI47" s="11">
         <f t="shared" si="12"/>
-        <v>368819</v>
+        <v>368848</v>
       </c>
       <c r="AJ47" s="13">
         <f>SUM(AJ9:AJ46)</f>
-        <v>2853750</v>
+        <v>2853779</v>
       </c>
       <c r="AK47" s="12">
         <f t="shared" si="13"/>
-        <v>0.86669205622633394</v>
+        <v>0.86670086360947218</v>
       </c>
       <c r="AL47" s="13">
         <f>SUM(AL9:AL46)</f>
@@ -7236,15 +7236,15 @@
       </c>
       <c r="AN47" s="11">
         <f t="shared" si="14"/>
-        <v>405277</v>
+        <v>405305</v>
       </c>
       <c r="AO47" s="13">
         <f>SUM(AO9:AO46)</f>
-        <v>2878452</v>
+        <v>2878480</v>
       </c>
       <c r="AP47" s="12">
         <f t="shared" si="15"/>
-        <v>0.86106176953612268</v>
+        <v>0.86107014547205873</v>
       </c>
       <c r="AQ47" s="13">
         <f>SUM(AQ9:AQ46)</f>
@@ -7256,15 +7256,15 @@
       </c>
       <c r="AS47" s="11">
         <f t="shared" si="16"/>
-        <v>1762950</v>
+        <v>1763003</v>
       </c>
       <c r="AT47" s="13">
         <f>SUM(AT9:AT46)</f>
-        <v>7684653</v>
+        <v>7684706</v>
       </c>
       <c r="AU47" s="12">
         <f t="shared" si="17"/>
-        <v>0.90882054601944051</v>
+        <v>0.90882681403036292</v>
       </c>
     </row>
     <row r="48" spans="1:47" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
chore: sync GST statistics files 2026-09-01
</commit_message>
<xml_diff>
--- a/gstdatabase/GSTR-1-2017-2018.xlsx
+++ b/gstdatabase/GSTR-1-2017-2018.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GSTN\Krishnan Sir\Monthly Report\Jun-26\GST Statistics Downloads 31st May 26\Downloads\GSTR 1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GSTN\Krishnan Sir\Monthly Report\Jul-26\GST Statistics Downloads 31st Jul 26\Downloads\GSTR 1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C927B25A-E4B3-4959-B5BD-939701EE9DC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF840D9D-3AB6-4DA6-8FC4-6D525B75DBD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -182,10 +182,10 @@
     <t>Andaman and Nicobar Islands</t>
   </si>
   <si>
-    <t>Data Considered upto 30th Jun 2026</t>
+    <t>Data Considered upto 31st Jul 2026</t>
   </si>
   <si>
-    <t>Filing %age as on 30th Jun 2026</t>
+    <t>Filing %age as on 31st Jul 2026</t>
   </si>
 </sst>
 </file>
@@ -685,7 +685,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AV58"/>
+  <dimension ref="A1:AV56"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.44140625" customWidth="1"/>
@@ -1031,14 +1031,14 @@
       </c>
       <c r="O9" s="9">
         <f>P9-N9</f>
-        <v>10923</v>
+        <v>10924</v>
       </c>
       <c r="P9" s="22">
-        <v>55853</v>
+        <v>55854</v>
       </c>
       <c r="Q9" s="10">
         <f>P9/M9</f>
-        <v>0.89324782497441146</v>
+        <v>0.89326381780962127</v>
       </c>
       <c r="R9" s="6">
         <v>25413</v>
@@ -1133,14 +1133,14 @@
       </c>
       <c r="AS9" s="9">
         <f>AT9-AR9</f>
-        <v>17928</v>
+        <v>17929</v>
       </c>
       <c r="AT9" s="22">
-        <v>62543</v>
+        <v>62544</v>
       </c>
       <c r="AU9" s="10">
         <f>AT9/AQ9</f>
-        <v>0.87178879580713953</v>
+        <v>0.87180273483781934</v>
       </c>
       <c r="AV9" s="7"/>
     </row>
@@ -1642,14 +1642,14 @@
       </c>
       <c r="E13" s="9">
         <f t="shared" si="0"/>
-        <v>16195</v>
+        <v>16198</v>
       </c>
       <c r="F13" s="22">
-        <v>75594</v>
+        <v>75597</v>
       </c>
       <c r="G13" s="10">
         <f t="shared" si="1"/>
-        <v>0.88548670493147474</v>
+        <v>0.88552184608176177</v>
       </c>
       <c r="H13" s="6">
         <v>34516</v>
@@ -1659,14 +1659,14 @@
       </c>
       <c r="J13" s="9">
         <f t="shared" si="2"/>
-        <v>2894</v>
+        <v>2896</v>
       </c>
       <c r="K13" s="22">
-        <v>26007</v>
+        <v>26009</v>
       </c>
       <c r="L13" s="10">
         <f t="shared" si="3"/>
-        <v>0.75347664851083551</v>
+        <v>0.75353459265268286</v>
       </c>
       <c r="M13" s="6">
         <v>100078</v>
@@ -1676,14 +1676,14 @@
       </c>
       <c r="O13" s="9">
         <f t="shared" si="4"/>
-        <v>21062</v>
+        <v>21064</v>
       </c>
       <c r="P13" s="22">
-        <v>87512</v>
+        <v>87514</v>
       </c>
       <c r="Q13" s="10">
         <f t="shared" si="5"/>
-        <v>0.87443793840804174</v>
+        <v>0.8744579228202003</v>
       </c>
       <c r="R13" s="6">
         <v>34094</v>
@@ -1693,14 +1693,14 @@
       </c>
       <c r="T13" s="9">
         <f t="shared" si="6"/>
-        <v>3417</v>
+        <v>3418</v>
       </c>
       <c r="U13" s="22">
-        <v>26820</v>
+        <v>26821</v>
       </c>
       <c r="V13" s="10">
         <f t="shared" si="7"/>
-        <v>0.7866486771866017</v>
+        <v>0.78667800786062059</v>
       </c>
       <c r="W13" s="6">
         <v>34556</v>
@@ -1710,14 +1710,14 @@
       </c>
       <c r="Y13" s="9">
         <f t="shared" si="8"/>
-        <v>3914</v>
+        <v>3915</v>
       </c>
       <c r="Z13" s="22">
-        <v>27527</v>
+        <v>27528</v>
       </c>
       <c r="AA13" s="10">
         <f t="shared" si="9"/>
-        <v>0.79659104062970254</v>
+        <v>0.79661997916425509</v>
       </c>
       <c r="AB13" s="6">
         <v>99756</v>
@@ -1744,14 +1744,14 @@
       </c>
       <c r="AI13" s="9">
         <f t="shared" si="12"/>
-        <v>4639</v>
+        <v>4640</v>
       </c>
       <c r="AJ13" s="22">
-        <v>27779</v>
+        <v>27780</v>
       </c>
       <c r="AK13" s="10">
         <f t="shared" si="13"/>
-        <v>0.77998034536010108</v>
+        <v>0.78000842341709953</v>
       </c>
       <c r="AL13" s="6">
         <v>36218</v>
@@ -2227,14 +2227,14 @@
       </c>
       <c r="AI16" s="9">
         <f t="shared" si="12"/>
-        <v>8641</v>
+        <v>8642</v>
       </c>
       <c r="AJ16" s="22">
-        <v>107468</v>
+        <v>107469</v>
       </c>
       <c r="AK16" s="10">
         <f t="shared" si="13"/>
-        <v>0.88419736225039702</v>
+        <v>0.88420558979126729</v>
       </c>
       <c r="AL16" s="6">
         <v>122081</v>
@@ -2244,14 +2244,14 @@
       </c>
       <c r="AN16" s="9">
         <f t="shared" si="14"/>
-        <v>9228</v>
+        <v>9229</v>
       </c>
       <c r="AO16" s="22">
-        <v>107666</v>
+        <v>107667</v>
       </c>
       <c r="AP16" s="10">
         <f t="shared" si="15"/>
-        <v>0.88192265790745483</v>
+        <v>0.88193084919029174</v>
       </c>
       <c r="AQ16" s="6">
         <v>455889</v>
@@ -2261,14 +2261,14 @@
       </c>
       <c r="AS16" s="9">
         <f t="shared" si="16"/>
-        <v>94223</v>
+        <v>94226</v>
       </c>
       <c r="AT16" s="22">
-        <v>430118</v>
+        <v>430121</v>
       </c>
       <c r="AU16" s="10">
         <f t="shared" si="17"/>
-        <v>0.94347088874704155</v>
+        <v>0.94347746929625409</v>
       </c>
     </row>
     <row r="17" spans="1:47" x14ac:dyDescent="0.3">
@@ -2320,14 +2320,14 @@
       </c>
       <c r="O17" s="9">
         <f t="shared" si="4"/>
-        <v>168607</v>
+        <v>168609</v>
       </c>
       <c r="P17" s="22">
-        <v>800815</v>
+        <v>800817</v>
       </c>
       <c r="Q17" s="10">
         <f t="shared" si="5"/>
-        <v>0.90196495828152312</v>
+        <v>0.90196721089906473</v>
       </c>
       <c r="R17" s="6">
         <v>272330</v>
@@ -2337,14 +2337,14 @@
       </c>
       <c r="T17" s="9">
         <f t="shared" si="6"/>
-        <v>23001</v>
+        <v>23002</v>
       </c>
       <c r="U17" s="22">
-        <v>228340</v>
+        <v>228341</v>
       </c>
       <c r="V17" s="10">
         <f t="shared" si="7"/>
-        <v>0.83846803510446888</v>
+        <v>0.83847170712003816</v>
       </c>
       <c r="W17" s="6">
         <v>275780</v>
@@ -2354,14 +2354,14 @@
       </c>
       <c r="Y17" s="9">
         <f t="shared" si="8"/>
-        <v>28166</v>
+        <v>28167</v>
       </c>
       <c r="Z17" s="22">
-        <v>235986</v>
+        <v>235987</v>
       </c>
       <c r="AA17" s="10">
         <f t="shared" si="9"/>
-        <v>0.85570382188701144</v>
+        <v>0.85570744796576981</v>
       </c>
       <c r="AB17" s="6">
         <v>847512</v>
@@ -2371,14 +2371,14 @@
       </c>
       <c r="AD17" s="9">
         <f t="shared" si="10"/>
-        <v>170080</v>
+        <v>170082</v>
       </c>
       <c r="AE17" s="22">
-        <v>769909</v>
+        <v>769911</v>
       </c>
       <c r="AF17" s="10">
         <f t="shared" si="11"/>
-        <v>0.90843433485307579</v>
+        <v>0.90843669470166799</v>
       </c>
       <c r="AG17" s="6">
         <v>284469</v>
@@ -2388,14 +2388,14 @@
       </c>
       <c r="AI17" s="9">
         <f t="shared" si="12"/>
-        <v>31554</v>
+        <v>31555</v>
       </c>
       <c r="AJ17" s="22">
-        <v>236488</v>
+        <v>236489</v>
       </c>
       <c r="AK17" s="10">
         <f t="shared" si="13"/>
-        <v>0.83133135772263411</v>
+        <v>0.83133487304416298</v>
       </c>
       <c r="AL17" s="6">
         <v>289980</v>
@@ -2405,14 +2405,14 @@
       </c>
       <c r="AN17" s="9">
         <f t="shared" si="14"/>
-        <v>34826</v>
+        <v>34827</v>
       </c>
       <c r="AO17" s="22">
-        <v>238248</v>
+        <v>238249</v>
       </c>
       <c r="AP17" s="10">
         <f t="shared" si="15"/>
-        <v>0.82160148975791436</v>
+        <v>0.82160493827160497</v>
       </c>
       <c r="AQ17" s="6">
         <v>913159</v>
@@ -2422,14 +2422,14 @@
       </c>
       <c r="AS17" s="9">
         <f t="shared" si="16"/>
-        <v>211268</v>
+        <v>211270</v>
       </c>
       <c r="AT17" s="22">
-        <v>816221</v>
+        <v>816223</v>
       </c>
       <c r="AU17" s="10">
         <f t="shared" si="17"/>
-        <v>0.8938432408813799</v>
+        <v>0.89384543108045811</v>
       </c>
     </row>
     <row r="18" spans="1:47" x14ac:dyDescent="0.3">
@@ -2769,14 +2769,14 @@
       </c>
       <c r="E20" s="9">
         <f t="shared" si="0"/>
-        <v>697</v>
+        <v>698</v>
       </c>
       <c r="F20" s="22">
-        <v>3440</v>
+        <v>3441</v>
       </c>
       <c r="G20" s="10">
         <f t="shared" si="1"/>
-        <v>0.83841091883987329</v>
+        <v>0.83865464294418723</v>
       </c>
       <c r="H20" s="6">
         <v>2893</v>
@@ -2803,14 +2803,14 @@
       </c>
       <c r="O20" s="9">
         <f t="shared" si="4"/>
-        <v>1316</v>
+        <v>1317</v>
       </c>
       <c r="P20" s="22">
-        <v>4759</v>
+        <v>4760</v>
       </c>
       <c r="Q20" s="10">
         <f t="shared" si="5"/>
-        <v>0.78427818061964405</v>
+        <v>0.78444297956493081</v>
       </c>
       <c r="R20" s="6">
         <v>3316</v>
@@ -2854,14 +2854,14 @@
       </c>
       <c r="AD20" s="9">
         <f t="shared" si="10"/>
-        <v>1739</v>
+        <v>1740</v>
       </c>
       <c r="AE20" s="22">
-        <v>5399</v>
+        <v>5400</v>
       </c>
       <c r="AF20" s="10">
         <f t="shared" si="11"/>
-        <v>0.80521998508575687</v>
+        <v>0.80536912751677847</v>
       </c>
       <c r="AG20" s="6">
         <v>3592</v>
@@ -2905,14 +2905,14 @@
       </c>
       <c r="AS20" s="9">
         <f t="shared" si="16"/>
-        <v>2603</v>
+        <v>2604</v>
       </c>
       <c r="AT20" s="22">
-        <v>6177</v>
+        <v>6178</v>
       </c>
       <c r="AU20" s="10">
         <f t="shared" si="17"/>
-        <v>0.7652378592666006</v>
+        <v>0.76536174430128845</v>
       </c>
     </row>
     <row r="21" spans="1:47" x14ac:dyDescent="0.3">
@@ -3252,14 +3252,14 @@
       </c>
       <c r="E23" s="9">
         <f t="shared" si="0"/>
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="F23" s="22">
-        <v>2054</v>
+        <v>2056</v>
       </c>
       <c r="G23" s="10">
         <f t="shared" si="1"/>
-        <v>0.83802529579763363</v>
+        <v>0.83884128926968582</v>
       </c>
       <c r="H23" s="6">
         <v>1965</v>
@@ -3269,14 +3269,14 @@
       </c>
       <c r="J23" s="9">
         <f t="shared" si="2"/>
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="K23" s="22">
-        <v>1530</v>
+        <v>1532</v>
       </c>
       <c r="L23" s="10">
         <f t="shared" si="3"/>
-        <v>0.77862595419847325</v>
+        <v>0.77964376590330786</v>
       </c>
       <c r="M23" s="6">
         <v>3300</v>
@@ -3286,14 +3286,14 @@
       </c>
       <c r="O23" s="9">
         <f t="shared" si="4"/>
-        <v>552</v>
+        <v>554</v>
       </c>
       <c r="P23" s="22">
-        <v>2653</v>
+        <v>2655</v>
       </c>
       <c r="Q23" s="10">
         <f t="shared" si="5"/>
-        <v>0.80393939393939395</v>
+        <v>0.80454545454545456</v>
       </c>
       <c r="R23" s="6">
         <v>2275</v>
@@ -3303,14 +3303,14 @@
       </c>
       <c r="T23" s="9">
         <f t="shared" si="6"/>
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="U23" s="22">
-        <v>1725</v>
+        <v>1727</v>
       </c>
       <c r="V23" s="10">
         <f t="shared" si="7"/>
-        <v>0.75824175824175821</v>
+        <v>0.75912087912087911</v>
       </c>
       <c r="W23" s="6">
         <v>2370</v>
@@ -3320,14 +3320,14 @@
       </c>
       <c r="Y23" s="9">
         <f t="shared" si="8"/>
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="Z23" s="22">
-        <v>1774</v>
+        <v>1776</v>
       </c>
       <c r="AA23" s="10">
         <f t="shared" si="9"/>
-        <v>0.74852320675105488</v>
+        <v>0.74936708860759493</v>
       </c>
       <c r="AB23" s="6">
         <v>3748</v>
@@ -3337,14 +3337,14 @@
       </c>
       <c r="AD23" s="9">
         <f t="shared" si="10"/>
-        <v>688</v>
+        <v>690</v>
       </c>
       <c r="AE23" s="22">
-        <v>2972</v>
+        <v>2974</v>
       </c>
       <c r="AF23" s="10">
         <f t="shared" si="11"/>
-        <v>0.79295624332977588</v>
+        <v>0.79348986125933829</v>
       </c>
       <c r="AG23" s="6">
         <v>2479</v>
@@ -3354,14 +3354,14 @@
       </c>
       <c r="AI23" s="9">
         <f t="shared" si="12"/>
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="AJ23" s="22">
-        <v>1829</v>
+        <v>1830</v>
       </c>
       <c r="AK23" s="10">
         <f t="shared" si="13"/>
-        <v>0.7377974989915288</v>
+        <v>0.73820088745461876</v>
       </c>
       <c r="AL23" s="6">
         <v>2578</v>
@@ -3371,14 +3371,14 @@
       </c>
       <c r="AN23" s="9">
         <f t="shared" si="14"/>
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="AO23" s="22">
-        <v>1890</v>
+        <v>1891</v>
       </c>
       <c r="AP23" s="10">
         <f t="shared" si="15"/>
-        <v>0.73312645461598136</v>
+        <v>0.73351435221101624</v>
       </c>
       <c r="AQ23" s="6">
         <v>4048</v>
@@ -3388,14 +3388,14 @@
       </c>
       <c r="AS23" s="9">
         <f t="shared" si="16"/>
-        <v>810</v>
+        <v>811</v>
       </c>
       <c r="AT23" s="22">
-        <v>3119</v>
+        <v>3120</v>
       </c>
       <c r="AU23" s="10">
         <f t="shared" si="17"/>
-        <v>0.77050395256916993</v>
+        <v>0.77075098814229248</v>
       </c>
     </row>
     <row r="24" spans="1:47" x14ac:dyDescent="0.3">
@@ -3608,14 +3608,14 @@
       </c>
       <c r="O25" s="9">
         <f t="shared" si="4"/>
-        <v>3220</v>
+        <v>3221</v>
       </c>
       <c r="P25" s="22">
-        <v>11741</v>
+        <v>11742</v>
       </c>
       <c r="Q25" s="10">
         <f t="shared" si="5"/>
-        <v>0.79892487751769192</v>
+        <v>0.79899292324442028</v>
       </c>
       <c r="R25" s="6">
         <v>8161</v>
@@ -3625,14 +3625,14 @@
       </c>
       <c r="T25" s="9">
         <f t="shared" si="6"/>
-        <v>1600</v>
+        <v>1601</v>
       </c>
       <c r="U25" s="22">
-        <v>6009</v>
+        <v>6010</v>
       </c>
       <c r="V25" s="10">
         <f t="shared" si="7"/>
-        <v>0.73630682514397749</v>
+        <v>0.73642935914716334</v>
       </c>
       <c r="W25" s="6">
         <v>8403</v>
@@ -3642,14 +3642,14 @@
       </c>
       <c r="Y25" s="9">
         <f t="shared" si="8"/>
-        <v>1723</v>
+        <v>1724</v>
       </c>
       <c r="Z25" s="22">
-        <v>6240</v>
+        <v>6241</v>
       </c>
       <c r="AA25" s="10">
         <f t="shared" si="9"/>
-        <v>0.74259193145305247</v>
+        <v>0.74271093657027254</v>
       </c>
       <c r="AB25" s="6">
         <v>15398</v>
@@ -3659,14 +3659,14 @@
       </c>
       <c r="AD25" s="9">
         <f t="shared" si="10"/>
-        <v>3679</v>
+        <v>3680</v>
       </c>
       <c r="AE25" s="22">
-        <v>12356</v>
+        <v>12357</v>
       </c>
       <c r="AF25" s="10">
         <f t="shared" si="11"/>
-        <v>0.80244187556825564</v>
+        <v>0.80250681906741139</v>
       </c>
       <c r="AG25" s="6">
         <v>8752</v>
@@ -3676,14 +3676,14 @@
       </c>
       <c r="AI25" s="9">
         <f t="shared" si="12"/>
-        <v>1959</v>
+        <v>1961</v>
       </c>
       <c r="AJ25" s="22">
-        <v>6317</v>
+        <v>6319</v>
       </c>
       <c r="AK25" s="10">
         <f t="shared" si="13"/>
-        <v>0.72177787934186477</v>
+        <v>0.72200639853747717</v>
       </c>
       <c r="AL25" s="6">
         <v>8845</v>
@@ -3693,14 +3693,14 @@
       </c>
       <c r="AN25" s="9">
         <f t="shared" si="14"/>
-        <v>2104</v>
+        <v>2106</v>
       </c>
       <c r="AO25" s="22">
-        <v>6374</v>
+        <v>6376</v>
       </c>
       <c r="AP25" s="10">
         <f t="shared" si="15"/>
-        <v>0.72063312605992091</v>
+        <v>0.72085924250989264</v>
       </c>
       <c r="AQ25" s="6">
         <v>16327</v>
@@ -3710,14 +3710,14 @@
       </c>
       <c r="AS25" s="9">
         <f t="shared" si="16"/>
-        <v>4532</v>
+        <v>4534</v>
       </c>
       <c r="AT25" s="22">
-        <v>12934</v>
+        <v>12936</v>
       </c>
       <c r="AU25" s="10">
         <f t="shared" si="17"/>
-        <v>0.79218472468916523</v>
+        <v>0.79230722116739138</v>
       </c>
     </row>
     <row r="26" spans="1:47" x14ac:dyDescent="0.3">
@@ -4218,14 +4218,14 @@
       </c>
       <c r="E29" s="9">
         <f t="shared" si="0"/>
-        <v>25970</v>
+        <v>25971</v>
       </c>
       <c r="F29" s="22">
-        <v>122776</v>
+        <v>122777</v>
       </c>
       <c r="G29" s="10">
         <f t="shared" si="1"/>
-        <v>0.87775513851653264</v>
+        <v>0.87776228775692577</v>
       </c>
       <c r="H29" s="6">
         <v>57678</v>
@@ -4379,14 +4379,14 @@
       </c>
       <c r="E30" s="9">
         <f t="shared" si="0"/>
-        <v>16367</v>
+        <v>16370</v>
       </c>
       <c r="F30" s="22">
-        <v>72629</v>
+        <v>72632</v>
       </c>
       <c r="G30" s="10">
         <f t="shared" si="1"/>
-        <v>0.87086176093238532</v>
+        <v>0.87089773258672165</v>
       </c>
       <c r="H30" s="6">
         <v>37862</v>
@@ -4413,14 +4413,14 @@
       </c>
       <c r="O30" s="9">
         <f t="shared" si="4"/>
-        <v>20868</v>
+        <v>20870</v>
       </c>
       <c r="P30" s="22">
-        <v>81244</v>
+        <v>81246</v>
       </c>
       <c r="Q30" s="10">
         <f t="shared" si="5"/>
-        <v>0.86445420980390075</v>
+        <v>0.86447549024823633</v>
       </c>
       <c r="R30" s="6">
         <v>36736</v>
@@ -4464,14 +4464,14 @@
       </c>
       <c r="AD30" s="9">
         <f t="shared" si="10"/>
-        <v>21958</v>
+        <v>21960</v>
       </c>
       <c r="AE30" s="22">
-        <v>79610</v>
+        <v>79612</v>
       </c>
       <c r="AF30" s="10">
         <f t="shared" si="11"/>
-        <v>0.8754412395394614</v>
+        <v>0.87546323278753424</v>
       </c>
       <c r="AG30" s="6">
         <v>37890</v>
@@ -4481,14 +4481,14 @@
       </c>
       <c r="AI30" s="9">
         <f t="shared" si="12"/>
-        <v>5937</v>
+        <v>5938</v>
       </c>
       <c r="AJ30" s="22">
-        <v>30640</v>
+        <v>30641</v>
       </c>
       <c r="AK30" s="10">
         <f t="shared" si="13"/>
-        <v>0.80865663763525997</v>
+        <v>0.80868302982317231</v>
       </c>
       <c r="AL30" s="6">
         <v>37957</v>
@@ -4515,14 +4515,14 @@
       </c>
       <c r="AS30" s="9">
         <f t="shared" si="16"/>
-        <v>27515</v>
+        <v>27516</v>
       </c>
       <c r="AT30" s="22">
-        <v>81681</v>
+        <v>81682</v>
       </c>
       <c r="AU30" s="10">
         <f t="shared" si="17"/>
-        <v>0.86573254618490925</v>
+        <v>0.86574314513137396</v>
       </c>
     </row>
     <row r="31" spans="1:47" x14ac:dyDescent="0.3">
@@ -4540,14 +4540,14 @@
       </c>
       <c r="E31" s="9">
         <f t="shared" si="0"/>
-        <v>43652</v>
+        <v>43653</v>
       </c>
       <c r="F31" s="22">
-        <v>240844</v>
+        <v>240845</v>
       </c>
       <c r="G31" s="10">
         <f t="shared" si="1"/>
-        <v>0.93601442629067111</v>
+        <v>0.93601831268363211</v>
       </c>
       <c r="H31" s="6">
         <v>94897</v>
@@ -4701,14 +4701,14 @@
       </c>
       <c r="E32" s="9">
         <f t="shared" si="0"/>
-        <v>68664</v>
+        <v>68669</v>
       </c>
       <c r="F32" s="22">
-        <v>540586</v>
+        <v>540591</v>
       </c>
       <c r="G32" s="10">
         <f t="shared" si="1"/>
-        <v>0.95757069042174237</v>
+        <v>0.95757954720577321</v>
       </c>
       <c r="H32" s="6">
         <v>224696</v>
@@ -4718,14 +4718,14 @@
       </c>
       <c r="J32" s="9">
         <f t="shared" si="2"/>
-        <v>8458</v>
+        <v>8459</v>
       </c>
       <c r="K32" s="22">
-        <v>204578</v>
+        <v>204579</v>
       </c>
       <c r="L32" s="10">
         <f t="shared" si="3"/>
-        <v>0.91046569587353576</v>
+        <v>0.91047014633104284</v>
       </c>
       <c r="M32" s="6">
         <v>682019</v>
@@ -4735,14 +4735,14 @@
       </c>
       <c r="O32" s="9">
         <f t="shared" si="4"/>
-        <v>94830</v>
+        <v>94832</v>
       </c>
       <c r="P32" s="22">
-        <v>656099</v>
+        <v>656101</v>
       </c>
       <c r="Q32" s="10">
         <f t="shared" si="5"/>
-        <v>0.96199519368228747</v>
+        <v>0.96199812615191072</v>
       </c>
       <c r="R32" s="6">
         <v>225967</v>
@@ -4752,14 +4752,14 @@
       </c>
       <c r="T32" s="9">
         <f t="shared" si="6"/>
-        <v>9814</v>
+        <v>9815</v>
       </c>
       <c r="U32" s="22">
-        <v>212617</v>
+        <v>212618</v>
       </c>
       <c r="V32" s="10">
         <f t="shared" si="7"/>
-        <v>0.9409205768983967</v>
+        <v>0.94092500232334808</v>
       </c>
       <c r="W32" s="6">
         <v>228262</v>
@@ -4769,14 +4769,14 @@
       </c>
       <c r="Y32" s="9">
         <f t="shared" si="8"/>
-        <v>11705</v>
+        <v>11707</v>
       </c>
       <c r="Z32" s="22">
-        <v>216310</v>
+        <v>216312</v>
       </c>
       <c r="AA32" s="10">
         <f t="shared" si="9"/>
-        <v>0.94763911645389942</v>
+        <v>0.94764787831526931</v>
       </c>
       <c r="AB32" s="6">
         <v>698869</v>
@@ -4786,14 +4786,14 @@
       </c>
       <c r="AD32" s="9">
         <f t="shared" si="10"/>
-        <v>100364</v>
+        <v>100365</v>
       </c>
       <c r="AE32" s="22">
-        <v>678198</v>
+        <v>678199</v>
       </c>
       <c r="AF32" s="10">
         <f t="shared" si="11"/>
-        <v>0.97042221074335822</v>
+        <v>0.97042364162668537</v>
       </c>
       <c r="AG32" s="6">
         <v>232401</v>
@@ -4803,14 +4803,14 @@
       </c>
       <c r="AI32" s="9">
         <f t="shared" si="12"/>
-        <v>13770</v>
+        <v>13773</v>
       </c>
       <c r="AJ32" s="22">
-        <v>218609</v>
+        <v>218612</v>
       </c>
       <c r="AK32" s="10">
         <f t="shared" si="13"/>
-        <v>0.94065430011058471</v>
+        <v>0.94066720883300847</v>
       </c>
       <c r="AL32" s="6">
         <v>234200</v>
@@ -4820,14 +4820,14 @@
       </c>
       <c r="AN32" s="9">
         <f t="shared" si="14"/>
-        <v>14853</v>
+        <v>14855</v>
       </c>
       <c r="AO32" s="22">
-        <v>219621</v>
+        <v>219623</v>
       </c>
       <c r="AP32" s="10">
         <f t="shared" si="15"/>
-        <v>0.93774978650725871</v>
+        <v>0.93775832621690858</v>
       </c>
       <c r="AQ32" s="6">
         <v>733311</v>
@@ -4837,14 +4837,14 @@
       </c>
       <c r="AS32" s="9">
         <f t="shared" si="16"/>
-        <v>118433</v>
+        <v>118437</v>
       </c>
       <c r="AT32" s="22">
-        <v>708217</v>
+        <v>708221</v>
       </c>
       <c r="AU32" s="10">
         <f t="shared" si="17"/>
-        <v>0.9657798669323111</v>
+        <v>0.96578532164388642</v>
       </c>
     </row>
     <row r="33" spans="1:47" x14ac:dyDescent="0.3">
@@ -5184,14 +5184,14 @@
       </c>
       <c r="E35" s="9">
         <f t="shared" si="0"/>
-        <v>145166</v>
+        <v>145168</v>
       </c>
       <c r="F35" s="22">
-        <v>864302</v>
+        <v>864304</v>
       </c>
       <c r="G35" s="10">
         <f t="shared" si="1"/>
-        <v>0.94470385575565208</v>
+        <v>0.94470604180602735</v>
       </c>
       <c r="H35" s="6">
         <v>336894</v>
@@ -5218,14 +5218,14 @@
       </c>
       <c r="O35" s="9">
         <f t="shared" si="4"/>
-        <v>190492</v>
+        <v>190493</v>
       </c>
       <c r="P35" s="22">
-        <v>1004075</v>
+        <v>1004076</v>
       </c>
       <c r="Q35" s="10">
         <f t="shared" si="5"/>
-        <v>0.94677610983291216</v>
+        <v>0.94677705276656732</v>
       </c>
       <c r="R35" s="6">
         <v>338572</v>
@@ -5269,14 +5269,14 @@
       </c>
       <c r="AD35" s="9">
         <f t="shared" si="10"/>
-        <v>211149</v>
+        <v>211150</v>
       </c>
       <c r="AE35" s="22">
-        <v>1042458</v>
+        <v>1042459</v>
       </c>
       <c r="AF35" s="10">
         <f t="shared" si="11"/>
-        <v>0.95244786679628402</v>
+        <v>0.95244878045214998</v>
       </c>
       <c r="AG35" s="6">
         <v>348478</v>
@@ -5286,14 +5286,14 @@
       </c>
       <c r="AI35" s="9">
         <f t="shared" si="12"/>
-        <v>36075</v>
+        <v>36076</v>
       </c>
       <c r="AJ35" s="22">
-        <v>316479</v>
+        <v>316480</v>
       </c>
       <c r="AK35" s="10">
         <f t="shared" si="13"/>
-        <v>0.90817497804739467</v>
+        <v>0.90817784766900633</v>
       </c>
       <c r="AL35" s="6">
         <v>352081</v>
@@ -5303,14 +5303,14 @@
       </c>
       <c r="AN35" s="9">
         <f t="shared" si="14"/>
-        <v>39185</v>
+        <v>39186</v>
       </c>
       <c r="AO35" s="22">
-        <v>318225</v>
+        <v>318226</v>
       </c>
       <c r="AP35" s="10">
         <f t="shared" si="15"/>
-        <v>0.90384030947424032</v>
+        <v>0.90384314972974966</v>
       </c>
       <c r="AQ35" s="6">
         <v>1148243</v>
@@ -5320,14 +5320,14 @@
       </c>
       <c r="AS35" s="9">
         <f t="shared" si="16"/>
-        <v>254041</v>
+        <v>254042</v>
       </c>
       <c r="AT35" s="22">
-        <v>1087100</v>
+        <v>1087101</v>
       </c>
       <c r="AU35" s="10">
         <f t="shared" si="17"/>
-        <v>0.94675081842432307</v>
+        <v>0.94675168932011777</v>
       </c>
     </row>
     <row r="36" spans="1:47" x14ac:dyDescent="0.3">
@@ -5345,14 +5345,14 @@
       </c>
       <c r="E36" s="9">
         <f t="shared" si="0"/>
-        <v>76412</v>
+        <v>76415</v>
       </c>
       <c r="F36" s="22">
-        <v>460731</v>
+        <v>460734</v>
       </c>
       <c r="G36" s="10">
         <f t="shared" si="1"/>
-        <v>0.91522565240451559</v>
+        <v>0.9152316117972138</v>
       </c>
       <c r="H36" s="6">
         <v>312358</v>
@@ -5362,14 +5362,14 @@
       </c>
       <c r="J36" s="9">
         <f t="shared" si="2"/>
-        <v>32464</v>
+        <v>32466</v>
       </c>
       <c r="K36" s="22">
-        <v>276707</v>
+        <v>276709</v>
       </c>
       <c r="L36" s="10">
         <f t="shared" si="3"/>
-        <v>0.88586493702738522</v>
+        <v>0.88587133993686729</v>
       </c>
       <c r="M36" s="6">
         <v>553919</v>
@@ -5379,14 +5379,14 @@
       </c>
       <c r="O36" s="9">
         <f t="shared" si="4"/>
-        <v>94059</v>
+        <v>94063</v>
       </c>
       <c r="P36" s="22">
-        <v>494799</v>
+        <v>494803</v>
       </c>
       <c r="Q36" s="10">
         <f t="shared" si="5"/>
-        <v>0.89326959356873481</v>
+        <v>0.89327681484115906</v>
       </c>
       <c r="R36" s="6">
         <v>318679</v>
@@ -5396,14 +5396,14 @@
       </c>
       <c r="T36" s="9">
         <f t="shared" si="6"/>
-        <v>35614</v>
+        <v>35619</v>
       </c>
       <c r="U36" s="22">
-        <v>284069</v>
+        <v>284074</v>
       </c>
       <c r="V36" s="10">
         <f t="shared" si="7"/>
-        <v>0.89139541670458355</v>
+        <v>0.89141110647391264</v>
       </c>
       <c r="W36" s="6">
         <v>324721</v>
@@ -5413,14 +5413,14 @@
       </c>
       <c r="Y36" s="9">
         <f t="shared" si="8"/>
-        <v>38959</v>
+        <v>38964</v>
       </c>
       <c r="Z36" s="22">
-        <v>289575</v>
+        <v>289580</v>
       </c>
       <c r="AA36" s="10">
         <f t="shared" si="9"/>
-        <v>0.89176554642292927</v>
+        <v>0.89178094425676191</v>
       </c>
       <c r="AB36" s="6">
         <v>556414</v>
@@ -5430,14 +5430,14 @@
       </c>
       <c r="AD36" s="9">
         <f t="shared" si="10"/>
-        <v>102232</v>
+        <v>102239</v>
       </c>
       <c r="AE36" s="22">
-        <v>499759</v>
+        <v>499766</v>
       </c>
       <c r="AF36" s="10">
         <f t="shared" si="11"/>
-        <v>0.89817833483700982</v>
+        <v>0.89819091539752771</v>
       </c>
       <c r="AG36" s="6">
         <v>333690</v>
@@ -5447,14 +5447,14 @@
       </c>
       <c r="AI36" s="9">
         <f t="shared" si="12"/>
-        <v>47427</v>
+        <v>47433</v>
       </c>
       <c r="AJ36" s="22">
-        <v>293786</v>
+        <v>293792</v>
       </c>
       <c r="AK36" s="10">
         <f t="shared" si="13"/>
-        <v>0.88041595492822677</v>
+        <v>0.88043393568881301</v>
       </c>
       <c r="AL36" s="6">
         <v>339216</v>
@@ -5464,14 +5464,14 @@
       </c>
       <c r="AN36" s="9">
         <f t="shared" si="14"/>
-        <v>52337</v>
+        <v>52342</v>
       </c>
       <c r="AO36" s="22">
-        <v>296773</v>
+        <v>296778</v>
       </c>
       <c r="AP36" s="10">
         <f t="shared" si="15"/>
-        <v>0.87487913305976128</v>
+        <v>0.87489387293052212</v>
       </c>
       <c r="AQ36" s="6">
         <v>590015</v>
@@ -5481,14 +5481,14 @@
       </c>
       <c r="AS36" s="9">
         <f t="shared" si="16"/>
-        <v>131203</v>
+        <v>131211</v>
       </c>
       <c r="AT36" s="22">
-        <v>521185</v>
+        <v>521193</v>
       </c>
       <c r="AU36" s="10">
         <f t="shared" si="17"/>
-        <v>0.88334194893350171</v>
+        <v>0.88335550791081585</v>
       </c>
     </row>
     <row r="37" spans="1:47" x14ac:dyDescent="0.3">
@@ -5828,14 +5828,14 @@
       </c>
       <c r="E39" s="9">
         <f t="shared" si="0"/>
-        <v>27790</v>
+        <v>27794</v>
       </c>
       <c r="F39" s="22">
-        <v>207441</v>
+        <v>207445</v>
       </c>
       <c r="G39" s="10">
         <f t="shared" si="1"/>
-        <v>0.96068633353401567</v>
+        <v>0.96070485805585148</v>
       </c>
       <c r="H39" s="6">
         <v>127093</v>
@@ -5896,14 +5896,14 @@
       </c>
       <c r="Y39" s="9">
         <f t="shared" si="8"/>
-        <v>14731</v>
+        <v>14732</v>
       </c>
       <c r="Z39" s="22">
-        <v>123693</v>
+        <v>123694</v>
       </c>
       <c r="AA39" s="10">
         <f t="shared" si="9"/>
-        <v>0.95492970794636034</v>
+        <v>0.95493742810601323</v>
       </c>
       <c r="AB39" s="6">
         <v>234754</v>
@@ -5913,14 +5913,14 @@
       </c>
       <c r="AD39" s="9">
         <f t="shared" si="10"/>
-        <v>39524</v>
+        <v>39525</v>
       </c>
       <c r="AE39" s="22">
-        <v>224346</v>
+        <v>224347</v>
       </c>
       <c r="AF39" s="10">
         <f t="shared" si="11"/>
-        <v>0.95566422723361477</v>
+        <v>0.95566848701193585</v>
       </c>
       <c r="AG39" s="6">
         <v>132146</v>
@@ -5964,14 +5964,14 @@
       </c>
       <c r="AS39" s="9">
         <f t="shared" si="16"/>
-        <v>50862</v>
+        <v>50863</v>
       </c>
       <c r="AT39" s="22">
-        <v>233366</v>
+        <v>233367</v>
       </c>
       <c r="AU39" s="10">
         <f t="shared" si="17"/>
-        <v>0.94956482110668494</v>
+        <v>0.94956889010054479</v>
       </c>
     </row>
     <row r="40" spans="1:47" x14ac:dyDescent="0.3">
@@ -5989,14 +5989,14 @@
       </c>
       <c r="E40" s="9">
         <f t="shared" si="0"/>
-        <v>75604</v>
+        <v>75621</v>
       </c>
       <c r="F40" s="22">
-        <v>569451</v>
+        <v>569468</v>
       </c>
       <c r="G40" s="10">
         <f t="shared" si="1"/>
-        <v>0.91131698636187597</v>
+        <v>0.91134419219480656</v>
       </c>
       <c r="H40" s="6">
         <v>436886</v>
@@ -6006,14 +6006,14 @@
       </c>
       <c r="J40" s="9">
         <f t="shared" si="2"/>
-        <v>35818</v>
+        <v>35832</v>
       </c>
       <c r="K40" s="22">
-        <v>380995</v>
+        <v>381009</v>
       </c>
       <c r="L40" s="10">
         <f t="shared" si="3"/>
-        <v>0.87206960168098768</v>
+        <v>0.87210164665381817</v>
       </c>
       <c r="M40" s="6">
         <v>700632</v>
@@ -6023,14 +6023,14 @@
       </c>
       <c r="O40" s="9">
         <f t="shared" si="4"/>
-        <v>101870</v>
+        <v>101884</v>
       </c>
       <c r="P40" s="22">
-        <v>624999</v>
+        <v>625013</v>
       </c>
       <c r="Q40" s="10">
         <f t="shared" si="5"/>
-        <v>0.89205032028225939</v>
+        <v>0.89207030224140493</v>
       </c>
       <c r="R40" s="6">
         <v>444591</v>
@@ -6040,14 +6040,14 @@
       </c>
       <c r="T40" s="9">
         <f t="shared" si="6"/>
-        <v>39760</v>
+        <v>39773</v>
       </c>
       <c r="U40" s="22">
-        <v>390963</v>
+        <v>390976</v>
       </c>
       <c r="V40" s="10">
         <f t="shared" si="7"/>
-        <v>0.8793767755082762</v>
+        <v>0.8794060158662681</v>
       </c>
       <c r="W40" s="6">
         <v>452148</v>
@@ -6057,14 +6057,14 @@
       </c>
       <c r="Y40" s="9">
         <f t="shared" si="8"/>
-        <v>43487</v>
+        <v>43501</v>
       </c>
       <c r="Z40" s="22">
-        <v>397636</v>
+        <v>397650</v>
       </c>
       <c r="AA40" s="10">
         <f t="shared" si="9"/>
-        <v>0.8794377062377805</v>
+        <v>0.87946866955067815</v>
       </c>
       <c r="AB40" s="6">
         <v>712131</v>
@@ -6074,14 +6074,14 @@
       </c>
       <c r="AD40" s="9">
         <f t="shared" si="10"/>
-        <v>112242</v>
+        <v>112256</v>
       </c>
       <c r="AE40" s="22">
-        <v>635555</v>
+        <v>635569</v>
       </c>
       <c r="AF40" s="10">
         <f t="shared" si="11"/>
-        <v>0.8924692226570673</v>
+        <v>0.89248888196132448</v>
       </c>
       <c r="AG40" s="6">
         <v>463481</v>
@@ -6091,14 +6091,14 @@
       </c>
       <c r="AI40" s="9">
         <f t="shared" si="12"/>
-        <v>52783</v>
+        <v>52794</v>
       </c>
       <c r="AJ40" s="22">
-        <v>402862</v>
+        <v>402873</v>
       </c>
       <c r="AK40" s="10">
         <f t="shared" si="13"/>
-        <v>0.86920930955098485</v>
+        <v>0.86923304299421122</v>
       </c>
       <c r="AL40" s="6">
         <v>472374</v>
@@ -6108,14 +6108,14 @@
       </c>
       <c r="AN40" s="9">
         <f t="shared" si="14"/>
-        <v>58007</v>
+        <v>58021</v>
       </c>
       <c r="AO40" s="22">
-        <v>408063</v>
+        <v>408077</v>
       </c>
       <c r="AP40" s="10">
         <f t="shared" si="15"/>
-        <v>0.86385575836095974</v>
+        <v>0.86388539589393154</v>
       </c>
       <c r="AQ40" s="6">
         <v>750910</v>
@@ -6125,14 +6125,14 @@
       </c>
       <c r="AS40" s="9">
         <f t="shared" si="16"/>
-        <v>138990</v>
+        <v>139006</v>
       </c>
       <c r="AT40" s="22">
-        <v>659148</v>
+        <v>659164</v>
       </c>
       <c r="AU40" s="10">
         <f t="shared" si="17"/>
-        <v>0.87779893728942215</v>
+        <v>0.87782024476967946</v>
       </c>
     </row>
     <row r="41" spans="1:47" x14ac:dyDescent="0.3">
@@ -6769,14 +6769,14 @@
       </c>
       <c r="AS44" s="9">
         <f t="shared" si="16"/>
-        <v>45592</v>
+        <v>45593</v>
       </c>
       <c r="AT44" s="22">
-        <v>201461</v>
+        <v>201462</v>
       </c>
       <c r="AU44" s="10">
         <f t="shared" si="17"/>
-        <v>0.88894232890614655</v>
+        <v>0.8889467413846357</v>
       </c>
     </row>
     <row r="45" spans="1:47" x14ac:dyDescent="0.3">
@@ -7096,15 +7096,15 @@
       </c>
       <c r="E47" s="11">
         <f>F47-D47</f>
-        <v>989563</v>
+        <v>989605</v>
       </c>
       <c r="F47" s="13">
         <f>SUM(F9:F46)</f>
-        <v>6283566</v>
+        <v>6283608</v>
       </c>
       <c r="G47" s="12">
         <f>F47/C47</f>
-        <v>0.92628931381308621</v>
+        <v>0.92629550522592097</v>
       </c>
       <c r="H47" s="13">
         <f>SUM(H9:H46)</f>
@@ -7116,15 +7116,15 @@
       </c>
       <c r="J47" s="11">
         <f t="shared" si="2"/>
-        <v>240263</v>
+        <v>240284</v>
       </c>
       <c r="K47" s="13">
         <f>SUM(K9:K46)</f>
-        <v>2669789</v>
+        <v>2669810</v>
       </c>
       <c r="L47" s="12">
         <f t="shared" si="3"/>
-        <v>0.84822094629542788</v>
+        <v>0.84822761822338633</v>
       </c>
       <c r="M47" s="13">
         <f>SUM(M9:M46)</f>
@@ -7136,15 +7136,15 @@
       </c>
       <c r="O47" s="11">
         <f t="shared" si="4"/>
-        <v>1297161</v>
+        <v>1297193</v>
       </c>
       <c r="P47" s="13">
         <f>SUM(P9:P46)</f>
-        <v>7192205</v>
+        <v>7192237</v>
       </c>
       <c r="Q47" s="12">
         <f t="shared" si="5"/>
-        <v>0.91771992399678604</v>
+        <v>0.91772400717260871</v>
       </c>
       <c r="R47" s="13">
         <f>SUM(R9:R46)</f>
@@ -7156,15 +7156,15 @@
       </c>
       <c r="T47" s="11">
         <f t="shared" si="6"/>
-        <v>273652</v>
+        <v>273676</v>
       </c>
       <c r="U47" s="13">
         <f>SUM(U9:U46)</f>
-        <v>2762785</v>
+        <v>2762809</v>
       </c>
       <c r="V47" s="12">
         <f t="shared" si="7"/>
-        <v>0.87430430752589972</v>
+        <v>0.87431190250827462</v>
       </c>
       <c r="W47" s="13">
         <f>SUM(W9:W46)</f>
@@ -7176,15 +7176,15 @@
       </c>
       <c r="Y47" s="11">
         <f t="shared" si="8"/>
-        <v>309642</v>
+        <v>309669</v>
       </c>
       <c r="Z47" s="13">
         <f>SUM(Z9:Z46)</f>
-        <v>2821196</v>
+        <v>2821223</v>
       </c>
       <c r="AA47" s="12">
         <f t="shared" si="9"/>
-        <v>0.87845472458107376</v>
+        <v>0.87846313175220392</v>
       </c>
       <c r="AB47" s="13">
         <f>SUM(AB9:AB46)</f>
@@ -7196,15 +7196,15 @@
       </c>
       <c r="AD47" s="11">
         <f t="shared" si="10"/>
-        <v>1416851</v>
+        <v>1416883</v>
       </c>
       <c r="AE47" s="13">
         <f>SUM(AE9:AE46)</f>
-        <v>7335721</v>
+        <v>7335753</v>
       </c>
       <c r="AF47" s="12">
         <f t="shared" si="11"/>
-        <v>0.92031553370043639</v>
+        <v>0.92031954831564311</v>
       </c>
       <c r="AG47" s="13">
         <f>SUM(AG9:AG46)</f>
@@ -7216,15 +7216,15 @@
       </c>
       <c r="AI47" s="11">
         <f t="shared" si="12"/>
-        <v>368848</v>
+        <v>368876</v>
       </c>
       <c r="AJ47" s="13">
         <f>SUM(AJ9:AJ46)</f>
-        <v>2853779</v>
+        <v>2853807</v>
       </c>
       <c r="AK47" s="12">
         <f t="shared" si="13"/>
-        <v>0.86670086360947218</v>
+        <v>0.86670936728974346</v>
       </c>
       <c r="AL47" s="13">
         <f>SUM(AL9:AL46)</f>
@@ -7236,15 +7236,15 @@
       </c>
       <c r="AN47" s="11">
         <f t="shared" si="14"/>
-        <v>405305</v>
+        <v>405332</v>
       </c>
       <c r="AO47" s="13">
         <f>SUM(AO9:AO46)</f>
-        <v>2878480</v>
+        <v>2878507</v>
       </c>
       <c r="AP47" s="12">
         <f t="shared" si="15"/>
-        <v>0.86107014547205873</v>
+        <v>0.8610782222674257</v>
       </c>
       <c r="AQ47" s="13">
         <f>SUM(AQ9:AQ46)</f>
@@ -7256,15 +7256,15 @@
       </c>
       <c r="AS47" s="11">
         <f t="shared" si="16"/>
-        <v>1763003</v>
+        <v>1763045</v>
       </c>
       <c r="AT47" s="13">
         <f>SUM(AT9:AT46)</f>
-        <v>7684706</v>
+        <v>7684748</v>
       </c>
       <c r="AU47" s="12">
         <f t="shared" si="17"/>
-        <v>0.90882681403036292</v>
+        <v>0.90883178113335805</v>
       </c>
     </row>
     <row r="48" spans="1:47" x14ac:dyDescent="0.3">
@@ -7345,74 +7345,52 @@
       <c r="AU54"/>
     </row>
     <row r="55" spans="1:47" x14ac:dyDescent="0.3">
-      <c r="G55"/>
-      <c r="L55"/>
-      <c r="Q55"/>
-      <c r="V55"/>
-      <c r="AA55"/>
-      <c r="AF55"/>
-      <c r="AK55"/>
-      <c r="AP55"/>
-      <c r="AU55"/>
+      <c r="C55" s="4"/>
+      <c r="D55" s="4"/>
+      <c r="E55" s="4"/>
+      <c r="F55" s="4"/>
+      <c r="H55" s="4"/>
+      <c r="I55" s="4"/>
+      <c r="J55" s="4"/>
+      <c r="K55" s="4"/>
+      <c r="M55" s="4"/>
+      <c r="N55" s="4"/>
+      <c r="O55" s="4"/>
+      <c r="P55" s="4"/>
+      <c r="R55" s="4"/>
+      <c r="S55" s="4"/>
+      <c r="T55" s="4"/>
+      <c r="U55" s="4"/>
+      <c r="W55" s="4"/>
+      <c r="X55" s="4"/>
+      <c r="Y55" s="4"/>
+      <c r="Z55" s="4"/>
+      <c r="AB55" s="4"/>
+      <c r="AC55" s="4"/>
+      <c r="AD55" s="4"/>
+      <c r="AE55" s="4"/>
+      <c r="AG55" s="4"/>
+      <c r="AH55" s="4"/>
+      <c r="AI55" s="4"/>
+      <c r="AJ55" s="4"/>
+      <c r="AL55" s="4"/>
+      <c r="AM55" s="4"/>
+      <c r="AN55" s="4"/>
+      <c r="AO55" s="4"/>
+      <c r="AQ55" s="4"/>
+      <c r="AR55" s="4"/>
+      <c r="AS55" s="4"/>
+      <c r="AT55" s="4"/>
     </row>
     <row r="56" spans="1:47" x14ac:dyDescent="0.3">
-      <c r="G56"/>
-      <c r="L56"/>
-      <c r="Q56"/>
-      <c r="V56"/>
-      <c r="AA56"/>
-      <c r="AF56"/>
-      <c r="AK56"/>
-      <c r="AP56"/>
-      <c r="AU56"/>
-    </row>
-    <row r="57" spans="1:47" x14ac:dyDescent="0.3">
-      <c r="C57" s="4"/>
-      <c r="D57" s="4"/>
-      <c r="E57" s="4"/>
-      <c r="F57" s="4"/>
-      <c r="H57" s="4"/>
-      <c r="I57" s="4"/>
-      <c r="J57" s="4"/>
-      <c r="K57" s="4"/>
-      <c r="M57" s="4"/>
-      <c r="N57" s="4"/>
-      <c r="O57" s="4"/>
-      <c r="P57" s="4"/>
-      <c r="R57" s="4"/>
-      <c r="S57" s="4"/>
-      <c r="T57" s="4"/>
-      <c r="U57" s="4"/>
-      <c r="W57" s="4"/>
-      <c r="X57" s="4"/>
-      <c r="Y57" s="4"/>
-      <c r="Z57" s="4"/>
-      <c r="AB57" s="4"/>
-      <c r="AC57" s="4"/>
-      <c r="AD57" s="4"/>
-      <c r="AE57" s="4"/>
-      <c r="AG57" s="4"/>
-      <c r="AH57" s="4"/>
-      <c r="AI57" s="4"/>
-      <c r="AJ57" s="4"/>
-      <c r="AL57" s="4"/>
-      <c r="AM57" s="4"/>
-      <c r="AN57" s="4"/>
-      <c r="AO57" s="4"/>
-      <c r="AQ57" s="4"/>
-      <c r="AR57" s="4"/>
-      <c r="AS57" s="4"/>
-      <c r="AT57" s="4"/>
-    </row>
-    <row r="58" spans="1:47" x14ac:dyDescent="0.3">
-      <c r="A58" s="27" t="s">
+      <c r="A56" s="27" t="s">
         <v>43</v>
       </c>
-      <c r="B58" s="27"/>
-      <c r="C58" s="27"/>
-      <c r="D58" s="27"/>
-      <c r="E58" s="27"/>
-      <c r="F58" s="5"/>
+      <c r="B56" s="27"/>
+      <c r="C56" s="27"/>
+      <c r="D56" s="27"/>
+      <c r="E56" s="27"/>
+      <c r="F56" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="15">
@@ -7423,7 +7401,7 @@
     <mergeCell ref="C7:G7"/>
     <mergeCell ref="AQ7:AU7"/>
     <mergeCell ref="A47:B47"/>
-    <mergeCell ref="A58:E58"/>
+    <mergeCell ref="A56:E56"/>
     <mergeCell ref="M7:Q7"/>
     <mergeCell ref="R7:V7"/>
     <mergeCell ref="W7:AA7"/>

</xml_diff>